<commit_message>
chute and diserio corrections
</commit_message>
<xml_diff>
--- a/data/2026 GSMUD.xlsx
+++ b/data/2026 GSMUD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code Space\Git 2026 Grad\2026-Grad\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE55BCE-4D68-4DB9-925B-E4630921AD53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027EB726-55DC-47FB-B98A-5253AC41FE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DIRECTIONS" sheetId="9" r:id="rId1"/>
@@ -476,9 +476,6 @@
   </si>
   <si>
     <t>Elsa Chow</t>
-  </si>
-  <si>
-    <t>Will Chite</t>
   </si>
   <si>
     <t>Max Cinelli</t>
@@ -1518,6 +1515,9 @@
   <si>
     <t>Uh-zra - the "Uh" part is slower than "zra" and roll the r. "Kud-reech" - roll the r</t>
   </si>
+  <si>
+    <t>Will Chute</t>
+  </si>
 </sst>
 </file>
 
@@ -1785,7 +1785,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1878,7 +1878,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2202,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="24" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -2210,7 +2209,7 @@
         <v>30</v>
       </c>
       <c r="O3" s="24" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2221,7 +2220,7 @@
         <v>31</v>
       </c>
       <c r="O4" s="24" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -2232,7 +2231,7 @@
         <v>32</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2240,7 +2239,7 @@
         <v>33</v>
       </c>
       <c r="O6" s="24" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -2248,7 +2247,7 @@
         <v>34</v>
       </c>
       <c r="O7" s="24" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -2259,7 +2258,7 @@
         <v>35</v>
       </c>
       <c r="O8" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2267,7 +2266,7 @@
         <v>36</v>
       </c>
       <c r="O9" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -2275,7 +2274,7 @@
         <v>37</v>
       </c>
       <c r="O10" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2283,7 +2282,7 @@
         <v>38</v>
       </c>
       <c r="O11" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -2291,7 +2290,7 @@
         <v>39</v>
       </c>
       <c r="O12" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -2305,7 +2304,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -2319,7 +2318,7 @@
         <v>41</v>
       </c>
       <c r="O14" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -2330,10 +2329,10 @@
         <v>10</v>
       </c>
       <c r="N15" s="24" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O15" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -2344,10 +2343,10 @@
         <v>12</v>
       </c>
       <c r="N16" s="24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="O16" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -2358,10 +2357,10 @@
         <v>14</v>
       </c>
       <c r="N17" s="24" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O17" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -2372,7 +2371,7 @@
         <v>42</v>
       </c>
       <c r="O18" s="24" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -2449,7 +2448,7 @@
         <v>Abate</v>
       </c>
       <c r="F2" s="45" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -2501,7 +2500,7 @@
         <v>Abubakar</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2514,13 +2513,13 @@
         <v>Luis</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H5" t="s">
         <v>25</v>
@@ -2547,7 +2546,7 @@
         <v>Ahlert</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2568,7 +2567,7 @@
         <v>Aiello</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2610,7 +2609,7 @@
         <v>Amado</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2688,7 +2687,7 @@
         <v>Aquino</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2728,7 +2727,7 @@
         <v>Araujo</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2749,7 +2748,7 @@
         <v>Aretusi</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2827,7 +2826,7 @@
         <v>Batista</v>
       </c>
       <c r="F20" s="45" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2848,7 +2847,7 @@
         <v>Beaulieu</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2869,7 +2868,7 @@
         <v>Belfon</v>
       </c>
       <c r="F22" s="45" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2928,7 +2927,7 @@
         <v>Bhola</v>
       </c>
       <c r="F25" s="46" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2968,7 +2967,7 @@
         <v>Boucher</v>
       </c>
       <c r="F27" s="41" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3008,12 +3007,12 @@
         <v>Bowlin</v>
       </c>
       <c r="F29" s="41" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="45" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="40" t="str">
@@ -3200,7 +3199,7 @@
         <v>Carcione</v>
       </c>
       <c r="F39" s="41" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3262,7 +3261,7 @@
     </row>
     <row r="43" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="41" t="s">
-        <v>135</v>
+        <v>481</v>
       </c>
       <c r="B43" s="41"/>
       <c r="C43" s="40" t="str">
@@ -3275,13 +3274,13 @@
       </c>
       <c r="E43" s="40" t="str">
         <f t="shared" si="5"/>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="F43" s="41"/>
     </row>
     <row r="44" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="46" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B44" s="41"/>
       <c r="C44" s="40" t="str">
@@ -3300,7 +3299,7 @@
     </row>
     <row r="45" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="46" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B45" s="41"/>
       <c r="C45" s="40" t="str">
@@ -3316,12 +3315,12 @@
         <v>Cirrone</v>
       </c>
       <c r="F45" s="46" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="45" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B46" s="41"/>
       <c r="C46" s="40" t="str">
@@ -3340,7 +3339,7 @@
     </row>
     <row r="47" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B47" s="41"/>
       <c r="C47" s="40" t="str">
@@ -3359,7 +3358,7 @@
     </row>
     <row r="48" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B48" s="41"/>
       <c r="C48" s="40" t="str">
@@ -3378,7 +3377,7 @@
     </row>
     <row r="49" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="47" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B49" s="41"/>
       <c r="C49" s="40" t="str">
@@ -3397,7 +3396,7 @@
     </row>
     <row r="50" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="45" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B50" s="41"/>
       <c r="C50" s="40" t="str">
@@ -3413,12 +3412,12 @@
         <v>Comenos</v>
       </c>
       <c r="F50" s="45" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="41" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B51" s="41"/>
       <c r="C51" s="40" t="str">
@@ -3434,12 +3433,12 @@
         <v>Connelly</v>
       </c>
       <c r="F51" s="41" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="45" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B52" s="41"/>
       <c r="C52" s="40" t="str">
@@ -3458,7 +3457,7 @@
     </row>
     <row r="53" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B53" s="41"/>
       <c r="C53" s="40" t="str">
@@ -3474,12 +3473,12 @@
         <v>Connor</v>
       </c>
       <c r="F53" s="46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B54" s="41"/>
       <c r="C54" s="40" t="str">
@@ -3498,7 +3497,7 @@
     </row>
     <row r="55" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="41" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B55" s="41"/>
       <c r="C55" s="40" t="str">
@@ -3517,7 +3516,7 @@
     </row>
     <row r="56" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="45" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B56" s="41"/>
       <c r="C56" s="40" t="str">
@@ -3536,7 +3535,7 @@
     </row>
     <row r="57" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B57" s="41"/>
       <c r="C57" s="40" t="str">
@@ -3555,7 +3554,7 @@
     </row>
     <row r="58" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="45" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B58" s="41"/>
       <c r="C58" s="40" t="str">
@@ -3574,7 +3573,7 @@
     </row>
     <row r="59" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="46" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B59" s="41"/>
       <c r="C59" s="40" t="str">
@@ -3593,7 +3592,7 @@
     </row>
     <row r="60" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="46" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B60" s="41"/>
       <c r="C60" s="40" t="str">
@@ -3612,7 +3611,7 @@
     </row>
     <row r="61" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B61" s="41"/>
       <c r="C61" s="40" t="str">
@@ -3631,7 +3630,7 @@
     </row>
     <row r="62" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="45" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B62" s="41"/>
       <c r="C62" s="40" t="str">
@@ -3640,15 +3639,15 @@
       </c>
       <c r="D62" s="40"/>
       <c r="E62" s="49" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F62" s="45" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="47" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B63" s="41"/>
       <c r="C63" s="40" t="str">
@@ -3667,7 +3666,7 @@
     </row>
     <row r="64" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="45" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B64" s="41"/>
       <c r="C64" s="40" t="str">
@@ -3683,12 +3682,12 @@
         <v>Dean</v>
       </c>
       <c r="F64" s="45" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="41" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B65" s="41"/>
       <c r="C65" s="40" t="str">
@@ -3704,12 +3703,12 @@
         <v>Deji</v>
       </c>
       <c r="F65" s="41" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="45" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B66" s="41"/>
       <c r="C66" s="40" t="str">
@@ -3728,7 +3727,7 @@
     </row>
     <row r="67" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="41" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B67" s="41"/>
       <c r="C67" s="40" t="str">
@@ -3744,7 +3743,7 @@
         <v>DiDonato</v>
       </c>
       <c r="F67" s="41" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3754,11 +3753,11 @@
       <c r="B68" s="41"/>
       <c r="C68" s="40" t="str">
         <f t="shared" si="3"/>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="D68" s="40" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Joseph</v>
       </c>
       <c r="E68" s="40" t="str">
         <f t="shared" si="5"/>
@@ -3768,28 +3767,28 @@
     </row>
     <row r="69" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="41" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B69" s="41"/>
       <c r="C69" s="40" t="str">
         <f t="shared" ref="C69:C132" si="6">IF(ISERROR( FIND(",",TRIM(A69))),LEFT(TRIM(A69), FIND(" ",TRIM(A69))-1),MID(TRIM(A69),LEN(C69)+3,FIND(" ",TRIM(A69)&amp;" ",LEN(C69)+3)-LEN(C69)-2))</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="D69" s="40" t="str">
         <f t="shared" ref="D69:D132" si="7">IF(ISERROR(FIND(",",TRIM(A69))),IF(LEN(TRIM(A69))-LEN(SUBSTITUTE(TRIM(A69)," ",""))=2,MID(TRIM(A69),LEN(C69)+2,FIND(" ",TRIM(A69),LEN(C69)+2)-LEN(C69)-2),""),MID(TRIM(A69),3+LEN(C69)+LEN(E69),30))</f>
-        <v>Joseph</v>
+        <v/>
       </c>
       <c r="E69" s="40" t="str">
         <f t="shared" ref="E69:E132" si="8">IF(ISERROR(FIND(",",TRIM(A69))),MID(TRIM(A69),1+LEN(TRIM(A69))-LEN(SUBSTITUTE(TRIM(A69)," ",""))+LEN(C69)+LEN(D69),30),LEFT(TRIM(A69), FIND(",",TRIM(A69))-1))</f>
         <v>DiSerio</v>
       </c>
       <c r="F69" s="41" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="45" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B70" s="41"/>
       <c r="C70" s="40" t="str">
@@ -3805,12 +3804,12 @@
         <v>Donaghey</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="46" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B71" s="41"/>
       <c r="C71" s="40" t="str">
@@ -3829,7 +3828,7 @@
     </row>
     <row r="72" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B72" s="41"/>
       <c r="C72" s="40" t="str">
@@ -3837,18 +3836,18 @@
         <v>Alana</v>
       </c>
       <c r="D72" s="49" t="s">
+        <v>469</v>
+      </c>
+      <c r="E72" s="49" t="s">
         <v>470</v>
       </c>
-      <c r="E72" s="49" t="s">
-        <v>471</v>
-      </c>
       <c r="F72" s="46" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B73" s="41"/>
       <c r="C73" s="40" t="str">
@@ -3867,7 +3866,7 @@
     </row>
     <row r="74" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="46" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B74" s="41"/>
       <c r="C74" s="40" t="str">
@@ -3883,12 +3882,12 @@
         <v>DuRoss</v>
       </c>
       <c r="F74" s="46" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="46" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B75" s="41"/>
       <c r="C75" s="40" t="str">
@@ -3907,7 +3906,7 @@
     </row>
     <row r="76" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B76" s="41"/>
       <c r="C76" s="40" t="str">
@@ -3926,7 +3925,7 @@
     </row>
     <row r="77" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B77" s="41"/>
       <c r="C77" s="40" t="str">
@@ -3945,7 +3944,7 @@
     </row>
     <row r="78" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="45" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B78" s="41"/>
       <c r="C78" s="40" t="str">
@@ -3964,7 +3963,7 @@
     </row>
     <row r="79" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B79" s="41"/>
       <c r="C79" s="40" t="str">
@@ -3983,7 +3982,7 @@
     </row>
     <row r="80" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="46" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B80" s="41"/>
       <c r="C80" s="40" t="str">
@@ -3999,12 +3998,12 @@
         <v>Encarnacao</v>
       </c>
       <c r="F80" s="46" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="46" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B81" s="41"/>
       <c r="C81" s="40" t="str">
@@ -4020,12 +4019,12 @@
         <v>Ewald</v>
       </c>
       <c r="F81" s="46" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="45" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B82" s="41"/>
       <c r="C82" s="40" t="str">
@@ -4041,12 +4040,12 @@
         <v>Fantasia</v>
       </c>
       <c r="F82" s="45" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="41" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B83" s="41"/>
       <c r="C83" s="40" t="str">
@@ -4065,7 +4064,7 @@
     </row>
     <row r="84" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B84" s="41"/>
       <c r="C84" s="40" t="str">
@@ -4084,7 +4083,7 @@
     </row>
     <row r="85" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="41" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B85" s="41"/>
       <c r="C85" s="40" t="str">
@@ -4103,7 +4102,7 @@
     </row>
     <row r="86" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="48" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B86" s="41"/>
       <c r="C86" s="40" t="str">
@@ -4122,7 +4121,7 @@
     </row>
     <row r="87" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="41" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B87" s="41"/>
       <c r="C87" s="40" t="str">
@@ -4141,7 +4140,7 @@
     </row>
     <row r="88" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="46" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B88" s="41"/>
       <c r="C88" s="40" t="str">
@@ -4160,7 +4159,7 @@
     </row>
     <row r="89" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="46" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B89" s="41"/>
       <c r="C89" s="40" t="str">
@@ -4176,12 +4175,12 @@
         <v>Forse</v>
       </c>
       <c r="F89" s="46" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="45" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B90" s="41"/>
       <c r="C90" s="40" t="str">
@@ -4200,7 +4199,7 @@
     </row>
     <row r="91" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B91" s="41"/>
       <c r="C91" s="40" t="str">
@@ -4219,7 +4218,7 @@
     </row>
     <row r="92" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B92" s="41"/>
       <c r="C92" s="40" t="str">
@@ -4235,12 +4234,12 @@
         <v>Fucarile</v>
       </c>
       <c r="F92" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B93" s="41"/>
       <c r="C93" s="40" t="str">
@@ -4259,7 +4258,7 @@
     </row>
     <row r="94" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="45" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B94" s="41"/>
       <c r="C94" s="40" t="str">
@@ -4278,7 +4277,7 @@
     </row>
     <row r="95" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="41" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B95" s="41"/>
       <c r="C95" s="40" t="str">
@@ -4294,12 +4293,12 @@
         <v>Gager</v>
       </c>
       <c r="F95" s="41" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A96" s="45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B96" s="41"/>
       <c r="C96" s="40" t="str">
@@ -4318,7 +4317,7 @@
     </row>
     <row r="97" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A97" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B97" s="41"/>
       <c r="C97" s="40" t="str">
@@ -4334,12 +4333,12 @@
         <v>Gallagher</v>
       </c>
       <c r="F97" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B98" s="41"/>
       <c r="C98" s="40" t="str">
@@ -4355,12 +4354,12 @@
         <v>Gauvin</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B99" s="41"/>
       <c r="C99" s="40" t="str">
@@ -4379,7 +4378,7 @@
     </row>
     <row r="100" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="46" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B100" s="41"/>
       <c r="C100" s="40" t="str">
@@ -4398,7 +4397,7 @@
     </row>
     <row r="101" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A101" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B101" s="41"/>
       <c r="C101" s="40" t="str">
@@ -4417,7 +4416,7 @@
     </row>
     <row r="102" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A102" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B102" s="41"/>
       <c r="C102" s="40" t="str">
@@ -4436,7 +4435,7 @@
     </row>
     <row r="103" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A103" s="46" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B103" s="41"/>
       <c r="C103" s="40" t="str">
@@ -4455,7 +4454,7 @@
     </row>
     <row r="104" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A104" s="46" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B104" s="41"/>
       <c r="C104" s="40" t="str">
@@ -4474,7 +4473,7 @@
     </row>
     <row r="105" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A105" s="41" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B105" s="41"/>
       <c r="C105" s="40" t="str">
@@ -4490,12 +4489,12 @@
         <v>Gorski</v>
       </c>
       <c r="F105" s="41" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A106" s="45" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B106" s="41"/>
       <c r="C106" s="40" t="str">
@@ -4511,12 +4510,12 @@
         <v>Gosdanian</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A107" s="46" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B107" s="41"/>
       <c r="C107" s="40" t="str">
@@ -4535,7 +4534,7 @@
     </row>
     <row r="108" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A108" s="46" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B108" s="41"/>
       <c r="C108" s="40" t="str">
@@ -4554,7 +4553,7 @@
     </row>
     <row r="109" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A109" s="41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B109" s="41"/>
       <c r="C109" s="40" t="str">
@@ -4573,7 +4572,7 @@
     </row>
     <row r="110" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A110" s="45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B110" s="41"/>
       <c r="C110" s="40" t="str">
@@ -4589,12 +4588,12 @@
         <v>Hall</v>
       </c>
       <c r="F110" s="45" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A111" s="41" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B111" s="41"/>
       <c r="C111" s="40" t="str">
@@ -4613,7 +4612,7 @@
     </row>
     <row r="112" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A112" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B112" s="41"/>
       <c r="C112" s="40" t="str">
@@ -4632,7 +4631,7 @@
     </row>
     <row r="113" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A113" s="47" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B113" s="41"/>
       <c r="C113" s="40" t="str">
@@ -4651,7 +4650,7 @@
     </row>
     <row r="114" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A114" s="45" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B114" s="41"/>
       <c r="C114" s="40" t="str">
@@ -4670,7 +4669,7 @@
     </row>
     <row r="115" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A115" s="46" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B115" s="41"/>
       <c r="C115" s="40" t="str">
@@ -4689,7 +4688,7 @@
     </row>
     <row r="116" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A116" s="46" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B116" s="41"/>
       <c r="C116" s="40" t="str">
@@ -4705,12 +4704,12 @@
         <v>Henri</v>
       </c>
       <c r="F116" s="46" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A117" s="41" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B117" s="41"/>
       <c r="C117" s="40" t="str">
@@ -4729,7 +4728,7 @@
     </row>
     <row r="118" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A118" s="46" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B118" s="41"/>
       <c r="C118" s="40" t="str">
@@ -4748,7 +4747,7 @@
     </row>
     <row r="119" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A119" s="41" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B119" s="41"/>
       <c r="C119" s="40" t="str">
@@ -4764,12 +4763,12 @@
         <v>Hobson</v>
       </c>
       <c r="F119" s="41" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A120" s="45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B120" s="41"/>
       <c r="C120" s="40" t="str">
@@ -4788,7 +4787,7 @@
     </row>
     <row r="121" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A121" s="46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B121" s="41"/>
       <c r="C121" s="40" t="str">
@@ -4804,12 +4803,12 @@
         <v>Houle</v>
       </c>
       <c r="F121" s="46" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A122" s="45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B122" s="41"/>
       <c r="C122" s="40" t="str">
@@ -4828,7 +4827,7 @@
     </row>
     <row r="123" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A123" s="41" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B123" s="41"/>
       <c r="C123" s="40" t="str">
@@ -4844,12 +4843,12 @@
         <v>Iosua</v>
       </c>
       <c r="F123" s="41" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A124" s="46" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B124" s="41"/>
       <c r="C124" s="40" t="str">
@@ -4868,7 +4867,7 @@
     </row>
     <row r="125" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A125" s="41" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B125" s="41"/>
       <c r="C125" s="40" t="str">
@@ -4887,7 +4886,7 @@
     </row>
     <row r="126" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A126" s="45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B126" s="41"/>
       <c r="C126" s="40" t="str">
@@ -4906,7 +4905,7 @@
     </row>
     <row r="127" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A127" s="41" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B127" s="41"/>
       <c r="C127" s="40" t="str">
@@ -4925,7 +4924,7 @@
     </row>
     <row r="128" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A128" s="46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B128" s="41"/>
       <c r="C128" s="40" t="str">
@@ -4944,7 +4943,7 @@
     </row>
     <row r="129" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A129" s="41" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B129" s="41"/>
       <c r="C129" s="40" t="str">
@@ -4963,7 +4962,7 @@
     </row>
     <row r="130" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A130" s="46" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B130" s="41"/>
       <c r="C130" s="40" t="str">
@@ -4982,7 +4981,7 @@
     </row>
     <row r="131" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A131" s="41" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B131" s="41"/>
       <c r="C131" s="40" t="str">
@@ -5001,7 +5000,7 @@
     </row>
     <row r="132" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A132" s="46" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B132" s="41"/>
       <c r="C132" s="40" t="str">
@@ -5017,12 +5016,12 @@
         <v>Kaberle</v>
       </c>
       <c r="F132" s="46" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A133" s="46" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B133" s="41"/>
       <c r="C133" s="40" t="str">
@@ -5038,12 +5037,12 @@
         <v>Kadric</v>
       </c>
       <c r="F133" s="46" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A134" s="45" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B134" s="41"/>
       <c r="C134" s="40" t="str">
@@ -5059,12 +5058,12 @@
         <v>Keaveney</v>
       </c>
       <c r="F134" s="45" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A135" s="46" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B135" s="41"/>
       <c r="C135" s="40" t="str">
@@ -5080,12 +5079,12 @@
         <v>Kenton</v>
       </c>
       <c r="F135" s="46" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A136" s="46" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B136" s="41"/>
       <c r="C136" s="40" t="str">
@@ -5101,12 +5100,12 @@
         <v>Kiley</v>
       </c>
       <c r="F136" s="46" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A137" s="41" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B137" s="41"/>
       <c r="C137" s="40" t="str">
@@ -5125,7 +5124,7 @@
     </row>
     <row r="138" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A138" s="45" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B138" s="41"/>
       <c r="C138" s="40" t="str">
@@ -5144,7 +5143,7 @@
     </row>
     <row r="139" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A139" s="41" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B139" s="41"/>
       <c r="C139" s="40" t="str">
@@ -5160,12 +5159,12 @@
         <v>Lalicata</v>
       </c>
       <c r="F139" s="41" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A140" s="45" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B140" s="41"/>
       <c r="C140" s="40" t="str">
@@ -5181,12 +5180,12 @@
         <v>Laurino</v>
       </c>
       <c r="F140" s="45" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="141" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A141" s="41" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B141" s="41"/>
       <c r="C141" s="40" t="str">
@@ -5205,7 +5204,7 @@
     </row>
     <row r="142" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A142" s="45" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B142" s="41"/>
       <c r="C142" s="40" t="str">
@@ -5221,12 +5220,12 @@
         <v>Layne</v>
       </c>
       <c r="F142" s="45" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A143" s="41" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B143" s="41"/>
       <c r="C143" s="40" t="str">
@@ -5245,7 +5244,7 @@
     </row>
     <row r="144" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A144" s="45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B144" s="41"/>
       <c r="C144" s="40" t="str">
@@ -5264,7 +5263,7 @@
     </row>
     <row r="145" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A145" s="41" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B145" s="41"/>
       <c r="C145" s="40" t="str">
@@ -5283,7 +5282,7 @@
     </row>
     <row r="146" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A146" s="45" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B146" s="41"/>
       <c r="C146" s="40" t="str">
@@ -5302,7 +5301,7 @@
     </row>
     <row r="147" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A147" s="41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B147" s="41"/>
       <c r="C147" s="40" t="str">
@@ -5321,7 +5320,7 @@
     </row>
     <row r="148" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A148" s="45" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B148" s="41"/>
       <c r="C148" s="40" t="str">
@@ -5340,7 +5339,7 @@
     </row>
     <row r="149" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A149" s="46" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B149" s="41"/>
       <c r="C149" s="40" t="str">
@@ -5356,12 +5355,12 @@
         <v>Lizotte</v>
       </c>
       <c r="F149" s="46" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A150" s="46" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B150" s="41"/>
       <c r="C150" s="40" t="str">
@@ -5377,12 +5376,12 @@
         <v>Lusk</v>
       </c>
       <c r="F150" s="46" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="151" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A151" s="46" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B151" s="41"/>
       <c r="C151" s="40" t="str">
@@ -5401,7 +5400,7 @@
     </row>
     <row r="152" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A152" s="45" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B152" s="41"/>
       <c r="C152" s="40" t="str">
@@ -5417,12 +5416,12 @@
         <v>Maganzini</v>
       </c>
       <c r="F152" s="45" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="153" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A153" s="41" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B153" s="41"/>
       <c r="C153" s="40" t="str">
@@ -5441,7 +5440,7 @@
     </row>
     <row r="154" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A154" s="45" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B154" s="41"/>
       <c r="C154" s="40" t="str">
@@ -5460,7 +5459,7 @@
     </row>
     <row r="155" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A155" s="41" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B155" s="41"/>
       <c r="C155" s="40" t="str">
@@ -5476,12 +5475,12 @@
         <v>Maness</v>
       </c>
       <c r="F155" s="41" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A156" s="45" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B156" s="41"/>
       <c r="C156" s="40" t="str">
@@ -5500,7 +5499,7 @@
     </row>
     <row r="157" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A157" s="41" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B157" s="41"/>
       <c r="C157" s="40" t="str">
@@ -5519,7 +5518,7 @@
     </row>
     <row r="158" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A158" s="46" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B158" s="41"/>
       <c r="C158" s="40" t="str">
@@ -5535,12 +5534,12 @@
         <v>Marchlik</v>
       </c>
       <c r="F158" s="46" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="159" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A159" s="41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B159" s="41"/>
       <c r="C159" s="40" t="e">
@@ -5556,12 +5555,12 @@
         <v>#VALUE!</v>
       </c>
       <c r="F159" s="41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="160" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A160" s="46" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B160" s="41"/>
       <c r="C160" s="40" t="str">
@@ -5580,7 +5579,7 @@
     </row>
     <row r="161" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A161" s="47" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B161" s="41"/>
       <c r="C161" s="40" t="str">
@@ -5599,7 +5598,7 @@
     </row>
     <row r="162" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A162" s="48" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B162" s="41"/>
       <c r="C162" s="40" t="str">
@@ -5618,7 +5617,7 @@
     </row>
     <row r="163" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A163" s="46" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B163" s="41"/>
       <c r="C163" s="40" t="str">
@@ -5637,7 +5636,7 @@
     </row>
     <row r="164" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A164" s="46" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B164" s="41"/>
       <c r="C164" s="40" t="str">
@@ -5656,7 +5655,7 @@
     </row>
     <row r="165" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A165" s="46" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B165" s="41"/>
       <c r="C165" s="40" t="str">
@@ -5675,7 +5674,7 @@
     </row>
     <row r="166" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A166" s="45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B166" s="41"/>
       <c r="C166" s="40" t="str">
@@ -5694,7 +5693,7 @@
     </row>
     <row r="167" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A167" s="41" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B167" s="41"/>
       <c r="C167" s="40" t="str">
@@ -5710,12 +5709,12 @@
         <v>McLaughlin-Shostak</v>
       </c>
       <c r="F167" s="41" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A168" s="45" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B168" s="41"/>
       <c r="C168" s="40" t="str">
@@ -5731,12 +5730,12 @@
         <v>McMenimen</v>
       </c>
       <c r="F168" s="45" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A169" s="41" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B169" s="41"/>
       <c r="C169" s="40" t="str">
@@ -5755,7 +5754,7 @@
     </row>
     <row r="170" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A170" s="46" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B170" s="41"/>
       <c r="C170" s="40" t="str">
@@ -5774,7 +5773,7 @@
     </row>
     <row r="171" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A171" s="46" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B171" s="41"/>
       <c r="C171" s="40" t="str">
@@ -5793,7 +5792,7 @@
     </row>
     <row r="172" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A172" s="46" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B172" s="41"/>
       <c r="C172" s="40" t="str">
@@ -5809,12 +5808,12 @@
         <v>Miceli</v>
       </c>
       <c r="F172" s="46" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="173" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A173" s="41" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B173" s="41"/>
       <c r="C173" s="40" t="str">
@@ -5833,7 +5832,7 @@
     </row>
     <row r="174" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A174" s="48" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B174" s="41"/>
       <c r="C174" s="40" t="str">
@@ -5852,7 +5851,7 @@
     </row>
     <row r="175" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A175" s="41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B175" s="41"/>
       <c r="C175" s="40" t="str">
@@ -5868,12 +5867,12 @@
         <v>Moller</v>
       </c>
       <c r="F175" s="41" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A176" s="45" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B176" s="41"/>
       <c r="C176" s="40" t="str">
@@ -5889,12 +5888,12 @@
         <v>Moreira</v>
       </c>
       <c r="F176" s="45" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A177" s="41" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B177" s="41"/>
       <c r="C177" s="40" t="str">
@@ -5913,7 +5912,7 @@
     </row>
     <row r="178" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A178" s="45" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B178" s="41"/>
       <c r="C178" s="40" t="str">
@@ -5932,7 +5931,7 @@
     </row>
     <row r="179" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A179" s="41" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B179" s="41"/>
       <c r="C179" s="40" t="str">
@@ -5951,7 +5950,7 @@
     </row>
     <row r="180" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A180" s="45" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B180" s="41"/>
       <c r="C180" s="40" t="str">
@@ -5967,12 +5966,12 @@
         <v>Muller</v>
       </c>
       <c r="F180" s="45" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A181" s="46" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B181" s="41"/>
       <c r="C181" s="40" t="str">
@@ -5988,7 +5987,7 @@
         <v>Mullin</v>
       </c>
       <c r="F181" s="46" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="182" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6012,7 +6011,7 @@
     </row>
     <row r="183" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A183" s="46" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B183" s="41"/>
       <c r="C183" s="40" t="str">
@@ -6031,7 +6030,7 @@
     </row>
     <row r="184" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A184" s="46" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B184" s="41"/>
       <c r="C184" s="40" t="str">
@@ -6050,7 +6049,7 @@
     </row>
     <row r="185" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A185" s="41" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B185" s="41"/>
       <c r="C185" s="40" t="str">
@@ -6066,12 +6065,12 @@
         <v>Nguyen</v>
       </c>
       <c r="F185" s="41" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="186" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A186" s="46" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B186" s="41"/>
       <c r="C186" s="40" t="str">
@@ -6090,7 +6089,7 @@
     </row>
     <row r="187" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A187" s="41" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B187" s="41"/>
       <c r="C187" s="40" t="str">
@@ -6106,12 +6105,12 @@
         <v>Norris</v>
       </c>
       <c r="F187" s="41" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="188" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A188" s="45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B188" s="41"/>
       <c r="C188" s="40" t="str">
@@ -6130,7 +6129,7 @@
     </row>
     <row r="189" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A189" s="41" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B189" s="41"/>
       <c r="C189" s="40" t="str">
@@ -6146,12 +6145,12 @@
         <v>Ortins</v>
       </c>
       <c r="F189" s="41" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="190" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A190" s="45" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B190" s="41"/>
       <c r="C190" s="40" t="str">
@@ -6167,12 +6166,12 @@
         <v>Ortiz</v>
       </c>
       <c r="F190" s="45" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="191" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A191" s="46" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B191" s="41"/>
       <c r="C191" s="40" t="str">
@@ -6191,7 +6190,7 @@
     </row>
     <row r="192" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A192" s="46" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B192" s="41"/>
       <c r="C192" s="40" t="str">
@@ -6207,12 +6206,12 @@
         <v>Patel</v>
       </c>
       <c r="F192" s="46" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A193" s="41" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B193" s="41"/>
       <c r="C193" s="40" t="str">
@@ -6231,7 +6230,7 @@
     </row>
     <row r="194" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A194" s="45" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B194" s="41"/>
       <c r="C194" s="40" t="str">
@@ -6247,12 +6246,12 @@
         <v>Petrin</v>
       </c>
       <c r="F194" s="45" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="195" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A195" s="41" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B195" s="41"/>
       <c r="C195" s="40" t="str">
@@ -6271,7 +6270,7 @@
     </row>
     <row r="196" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A196" s="48" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B196" s="41"/>
       <c r="C196" s="40" t="str">
@@ -6290,7 +6289,7 @@
     </row>
     <row r="197" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A197" s="46" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B197" s="41"/>
       <c r="C197" s="40" t="str">
@@ -6306,12 +6305,12 @@
         <v>Pomerantz</v>
       </c>
       <c r="F197" s="46" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="198" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A198" s="45" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B198" s="41"/>
       <c r="C198" s="40" t="str">
@@ -6327,12 +6326,12 @@
         <v>Poudyal</v>
       </c>
       <c r="F198" s="45" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="199" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A199" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B199" s="41"/>
       <c r="C199" s="40" t="str">
@@ -6348,12 +6347,12 @@
         <v>Pulpi</v>
       </c>
       <c r="F199" s="46" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="200" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A200" s="46" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B200" s="41"/>
       <c r="C200" s="40" t="str">
@@ -6369,12 +6368,12 @@
         <v>Rai</v>
       </c>
       <c r="F200" s="46" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="201" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A201" s="46" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B201" s="41"/>
       <c r="C201" s="40" t="str">
@@ -6393,7 +6392,7 @@
     </row>
     <row r="202" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A202" s="46" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B202" s="41"/>
       <c r="C202" s="40" t="str">
@@ -6412,7 +6411,7 @@
     </row>
     <row r="203" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A203" s="46" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B203" s="41"/>
       <c r="C203" s="40" t="str">
@@ -6431,7 +6430,7 @@
     </row>
     <row r="204" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A204" s="46" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B204" s="41"/>
       <c r="C204" s="40" t="str">
@@ -6447,12 +6446,12 @@
         <v>Richter</v>
       </c>
       <c r="F204" s="46" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="205" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A205" s="46" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B205" s="41"/>
       <c r="C205" s="40" t="str">
@@ -6468,12 +6467,12 @@
         <v>Robichaud</v>
       </c>
       <c r="F205" s="46" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="206" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A206" s="45" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B206" s="41"/>
       <c r="C206" s="40" t="str">
@@ -6492,7 +6491,7 @@
     </row>
     <row r="207" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A207" s="41" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B207" s="41"/>
       <c r="C207" s="40" t="str">
@@ -6511,7 +6510,7 @@
     </row>
     <row r="208" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A208" s="46" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B208" s="41"/>
       <c r="C208" s="40" t="str">
@@ -6530,7 +6529,7 @@
     </row>
     <row r="209" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A209" s="41" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B209" s="41"/>
       <c r="C209" s="40" t="str">
@@ -6549,7 +6548,7 @@
     </row>
     <row r="210" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A210" s="45" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B210" s="41"/>
       <c r="C210" s="40" t="str">
@@ -6568,7 +6567,7 @@
     </row>
     <row r="211" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A211" s="41" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B211" s="41"/>
       <c r="C211" s="40" t="str">
@@ -6584,12 +6583,12 @@
         <v>Rojas</v>
       </c>
       <c r="F211" s="41" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="212" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A212" s="46" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B212" s="41"/>
       <c r="C212" s="40" t="str">
@@ -6608,7 +6607,7 @@
     </row>
     <row r="213" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A213" s="41" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B213" s="41"/>
       <c r="C213" s="40" t="str">
@@ -6624,12 +6623,12 @@
         <v>Ryland</v>
       </c>
       <c r="F213" s="41" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="214" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A214" s="45" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B214" s="41"/>
       <c r="C214" s="40" t="str">
@@ -6645,12 +6644,12 @@
         <v>Sardinha</v>
       </c>
       <c r="F214" s="45" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="215" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A215" s="41" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B215" s="41"/>
       <c r="C215" s="40" t="str">
@@ -6666,12 +6665,12 @@
         <v>Sarre</v>
       </c>
       <c r="F215" s="41" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="216" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A216" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B216" s="41"/>
       <c r="C216" s="40" t="str">
@@ -6690,7 +6689,7 @@
     </row>
     <row r="217" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A217" s="41" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B217" s="41"/>
       <c r="C217" s="40" t="str">
@@ -6709,7 +6708,7 @@
     </row>
     <row r="218" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A218" s="45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B218" s="41"/>
       <c r="C218" s="40" t="str">
@@ -6725,12 +6724,12 @@
         <v>Schrager</v>
       </c>
       <c r="F218" s="45" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="219" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A219" s="41" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B219" s="41"/>
       <c r="C219" s="40" t="str">
@@ -6749,7 +6748,7 @@
     </row>
     <row r="220" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A220" s="45" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B220" s="41"/>
       <c r="C220" s="40" t="str">
@@ -6768,7 +6767,7 @@
     </row>
     <row r="221" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A221" s="46" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B221" s="41"/>
       <c r="C221" s="40" t="str">
@@ -6784,12 +6783,12 @@
         <v>Selvakumar</v>
       </c>
       <c r="F221" s="46" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="222" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A222" s="45" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B222" s="41"/>
       <c r="C222" s="40" t="str">
@@ -6808,7 +6807,7 @@
     </row>
     <row r="223" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A223" s="46" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B223" s="41"/>
       <c r="C223" s="40" t="str">
@@ -6827,7 +6826,7 @@
     </row>
     <row r="224" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A224" s="45" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B224" s="41"/>
       <c r="C224" s="40" t="str">
@@ -6843,12 +6842,12 @@
         <v>Shediac</v>
       </c>
       <c r="F224" s="45" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="225" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A225" s="41" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B225" s="41"/>
       <c r="C225" s="40" t="str">
@@ -6867,7 +6866,7 @@
     </row>
     <row r="226" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A226" s="45" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B226" s="41"/>
       <c r="C226" s="40" t="str">
@@ -6883,12 +6882,12 @@
         <v>Siciliano</v>
       </c>
       <c r="F226" s="45" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="227" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A227" s="46" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B227" s="41"/>
       <c r="C227" s="40" t="str">
@@ -6907,7 +6906,7 @@
     </row>
     <row r="228" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A228" s="46" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B228" s="41"/>
       <c r="C228" s="40" t="str">
@@ -6923,12 +6922,12 @@
         <v>Skenderian</v>
       </c>
       <c r="F228" s="46" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="229" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A229" s="41" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B229" s="41"/>
       <c r="C229" s="40" t="str">
@@ -6944,12 +6943,12 @@
         <v>Slinn</v>
       </c>
       <c r="F229" s="41" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="230" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A230" s="46" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B230" s="41"/>
       <c r="C230" s="40" t="str">
@@ -6968,7 +6967,7 @@
     </row>
     <row r="231" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A231" s="41" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B231" s="41"/>
       <c r="C231" s="40" t="str">
@@ -6987,7 +6986,7 @@
     </row>
     <row r="232" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A232" s="45" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B232" s="41"/>
       <c r="C232" s="40" t="str">
@@ -7003,12 +7002,12 @@
         <v>Soto</v>
       </c>
       <c r="F232" s="45" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="233" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A233" s="41" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B233" s="41"/>
       <c r="C233" s="40" t="str">
@@ -7027,7 +7026,7 @@
     </row>
     <row r="234" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A234" s="45" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B234" s="41"/>
       <c r="C234" s="40" t="str">
@@ -7046,7 +7045,7 @@
     </row>
     <row r="235" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A235" s="41" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B235" s="41"/>
       <c r="C235" s="40" t="str">
@@ -7065,7 +7064,7 @@
     </row>
     <row r="236" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A236" s="46" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B236" s="41"/>
       <c r="C236" s="40" t="str">
@@ -7081,12 +7080,12 @@
         <v>Staffier</v>
       </c>
       <c r="F236" s="46" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="237" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A237" s="46" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B237" s="41"/>
       <c r="C237" s="40" t="str">
@@ -7102,12 +7101,12 @@
         <v>Stathoulopoulos</v>
       </c>
       <c r="F237" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="238" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A238" s="45" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B238" s="41"/>
       <c r="C238" s="40" t="str">
@@ -7126,7 +7125,7 @@
     </row>
     <row r="239" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A239" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B239" s="41"/>
       <c r="C239" s="40" t="str">
@@ -7142,12 +7141,12 @@
         <v>Sullivan</v>
       </c>
       <c r="F239" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="240" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A240" s="46" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B240" s="41"/>
       <c r="C240" s="40" t="str">
@@ -7166,7 +7165,7 @@
     </row>
     <row r="241" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A241" s="41" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B241" s="41"/>
       <c r="C241" s="40" t="str">
@@ -7185,7 +7184,7 @@
     </row>
     <row r="242" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A242" s="45" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B242" s="41"/>
       <c r="C242" s="40" t="str">
@@ -7201,12 +7200,12 @@
         <v>Taubman</v>
       </c>
       <c r="F242" s="45" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="243" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A243" s="41" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B243" s="41"/>
       <c r="C243" s="40" t="str">
@@ -7222,12 +7221,12 @@
         <v>Tawadros</v>
       </c>
       <c r="F243" s="41" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="244" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A244" s="45" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B244" s="41"/>
       <c r="C244" s="40" t="str">
@@ -7243,12 +7242,12 @@
         <v>Toomey</v>
       </c>
       <c r="F244" s="45" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="245" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A245" s="41" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B245" s="41"/>
       <c r="C245" s="40" t="str">
@@ -7267,7 +7266,7 @@
     </row>
     <row r="246" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A246" s="45" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B246" s="41"/>
       <c r="C246" s="40" t="str">
@@ -7283,12 +7282,12 @@
         <v>Travassos</v>
       </c>
       <c r="F246" s="45" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="247" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A247" s="46" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B247" s="41"/>
       <c r="C247" s="40" t="str">
@@ -7304,12 +7303,12 @@
         <v>Upton</v>
       </c>
       <c r="F247" s="46" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="248" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A248" s="45" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B248" s="41"/>
       <c r="C248" s="40" t="str">
@@ -7328,7 +7327,7 @@
     </row>
     <row r="249" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A249" s="41" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B249" s="41"/>
       <c r="C249" s="40" t="str">
@@ -7337,13 +7336,13 @@
       </c>
       <c r="D249" s="40"/>
       <c r="E249" s="49" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F249" s="41"/>
     </row>
     <row r="250" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A250" s="45" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B250" s="41"/>
       <c r="C250" s="40" t="str">
@@ -7351,16 +7350,16 @@
         <v>Katherine</v>
       </c>
       <c r="D250" s="49" t="s">
+        <v>467</v>
+      </c>
+      <c r="E250" s="49" t="s">
         <v>468</v>
-      </c>
-      <c r="E250" s="49" t="s">
-        <v>469</v>
       </c>
       <c r="F250" s="45"/>
     </row>
     <row r="251" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A251" s="41" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B251" s="41"/>
       <c r="C251" s="40" t="str">
@@ -7379,7 +7378,7 @@
     </row>
     <row r="252" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A252" s="45" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B252" s="41"/>
       <c r="C252" s="40" t="str">
@@ -7395,12 +7394,12 @@
         <v>Viliott</v>
       </c>
       <c r="F252" s="45" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="253" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A253" s="46" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B253" s="41"/>
       <c r="C253" s="40" t="str">
@@ -7416,12 +7415,12 @@
         <v>Vitarisi</v>
       </c>
       <c r="F253" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="254" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A254" s="46" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B254" s="41"/>
       <c r="C254" s="40" t="str">
@@ -7440,7 +7439,7 @@
     </row>
     <row r="255" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A255" s="46" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B255" s="41"/>
       <c r="C255" s="40" t="str">
@@ -7459,7 +7458,7 @@
     </row>
     <row r="256" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A256" s="45" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B256" s="41"/>
       <c r="C256" s="40" t="str">
@@ -7478,7 +7477,7 @@
     </row>
     <row r="257" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A257" s="46" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B257" s="41"/>
       <c r="C257" s="40" t="str">
@@ -7497,7 +7496,7 @@
     </row>
     <row r="258" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A258" s="45" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B258" s="41"/>
       <c r="C258" s="40" t="str">
@@ -7516,7 +7515,7 @@
     </row>
     <row r="259" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A259" s="46" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B259" s="41"/>
       <c r="C259" s="40" t="str">
@@ -7535,7 +7534,7 @@
     </row>
     <row r="260" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A260" s="45" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B260" s="41"/>
       <c r="C260" s="40" t="str">
@@ -7554,7 +7553,7 @@
     </row>
     <row r="261" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A261" s="41" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B261" s="41"/>
       <c r="C261" s="40" t="str">
@@ -7573,7 +7572,7 @@
     </row>
     <row r="262" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A262" s="45" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B262" s="41"/>
       <c r="C262" s="40" t="str">
@@ -7592,7 +7591,7 @@
     </row>
     <row r="263" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A263" s="41" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B263" s="41"/>
       <c r="C263" s="40" t="str">
@@ -7608,12 +7607,12 @@
         <v>Williams</v>
       </c>
       <c r="F263" s="41" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="264" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A264" s="45" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B264" s="41"/>
       <c r="C264" s="40" t="str">
@@ -7632,7 +7631,7 @@
     </row>
     <row r="265" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A265" s="41" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C265" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7650,7 +7649,7 @@
     </row>
     <row r="266" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A266" s="45" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C266" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7668,7 +7667,7 @@
     </row>
     <row r="267" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A267" s="41" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C267" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7686,7 +7685,7 @@
     </row>
     <row r="268" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A268" s="45" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C268" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7701,12 +7700,12 @@
         <v>Zani</v>
       </c>
       <c r="F268" s="45" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="269" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A269" s="41" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C269" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7721,7 +7720,7 @@
         <v>Zheng</v>
       </c>
       <c r="F269" s="41" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.2">
@@ -7798,7 +7797,7 @@
       <c r="H2" s="42"/>
       <c r="I2" s="42"/>
       <c r="L2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -7829,7 +7828,7 @@
       <c r="H3" s="42"/>
       <c r="I3" s="42"/>
       <c r="L3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -7860,7 +7859,7 @@
       <c r="H4" s="42"/>
       <c r="I4" s="42"/>
       <c r="L4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -7891,7 +7890,7 @@
       <c r="H5" s="42"/>
       <c r="I5" s="42"/>
       <c r="L5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -7950,7 +7949,7 @@
       <c r="H7" s="42"/>
       <c r="I7" s="42"/>
       <c r="L7" s="22" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -7984,7 +7983,7 @@
         <v>30</v>
       </c>
       <c r="M8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -8018,7 +8017,7 @@
         <v>87</v>
       </c>
       <c r="M9" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -8052,7 +8051,7 @@
         <v>31</v>
       </c>
       <c r="M10" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -8086,7 +8085,7 @@
         <v>32</v>
       </c>
       <c r="M11" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -8120,7 +8119,7 @@
         <v>33</v>
       </c>
       <c r="M12" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -8154,7 +8153,7 @@
         <v>34</v>
       </c>
       <c r="M13" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -8188,7 +8187,7 @@
         <v>35</v>
       </c>
       <c r="M14" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -8222,7 +8221,7 @@
         <v>36</v>
       </c>
       <c r="M15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -8256,7 +8255,7 @@
         <v>37</v>
       </c>
       <c r="M16" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -8290,7 +8289,7 @@
         <v>38</v>
       </c>
       <c r="M17" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -8324,7 +8323,7 @@
         <v>39</v>
       </c>
       <c r="M18" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -8358,7 +8357,7 @@
         <v>40</v>
       </c>
       <c r="M19" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -8392,7 +8391,7 @@
         <v>41</v>
       </c>
       <c r="M20" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -8423,10 +8422,10 @@
       <c r="H21" s="42"/>
       <c r="I21" s="42"/>
       <c r="L21" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M21" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -8457,10 +8456,10 @@
       <c r="H22" s="42"/>
       <c r="I22" s="42"/>
       <c r="L22" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="M22" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -8491,10 +8490,10 @@
       <c r="H23" s="42"/>
       <c r="I23" s="42"/>
       <c r="L23" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="M23" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -8528,7 +8527,7 @@
         <v>42</v>
       </c>
       <c r="M24" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -9044,7 +9043,7 @@
       </c>
       <c r="E43" s="39" t="str">
         <f>'Raw Name Splitter'!E43</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="F43" s="39">
         <f>'Raw Name Splitter'!F43</f>
@@ -9730,11 +9729,11 @@
       </c>
       <c r="C68" s="39" t="str">
         <f>'Raw Name Splitter'!C68</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="D68" s="39" t="str">
         <f>'Raw Name Splitter'!D68</f>
-        <v/>
+        <v>Joseph</v>
       </c>
       <c r="E68" s="39" t="str">
         <f>'Raw Name Splitter'!E68</f>
@@ -9758,11 +9757,11 @@
       </c>
       <c r="C69" s="39" t="str">
         <f>'Raw Name Splitter'!C69</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="D69" s="39" t="str">
         <f>'Raw Name Splitter'!D69</f>
-        <v>Joseph</v>
+        <v/>
       </c>
       <c r="E69" s="39" t="str">
         <f>'Raw Name Splitter'!E69</f>
@@ -10099,7 +10098,7 @@
         <v/>
       </c>
       <c r="E81" s="39" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F81" s="39" t="str">
         <f>'Raw Name Splitter'!F81</f>
@@ -14772,7 +14771,7 @@
         <v>Colby</v>
       </c>
       <c r="E249" s="39" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F249" s="39">
         <f>'Raw Name Splitter'!F249</f>
@@ -15335,13 +15334,13 @@
         <v>87</v>
       </c>
       <c r="C270" s="39" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E270" s="39" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F270" s="39" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
   </sheetData>
@@ -17557,7 +17556,7 @@
       </c>
       <c r="H52" s="1" t="str">
         <f>VLOOKUP(J52,'Names with Seat Code'!A:E,5,FALSE)</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="I52" s="1" t="str">
         <f>VLOOKUP(J52,'Names with Seat Code'!A:E,3,FALSE)</f>
@@ -18507,14 +18506,14 @@
       </c>
       <c r="I74" s="1" t="str">
         <f>VLOOKUP(J74,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="J74" s="3">
         <v>61</v>
       </c>
       <c r="K74" t="str">
         <f>VLOOKUP(J74,'Names with Seat Code'!A:E,4,FALSE)</f>
-        <v/>
+        <v>Joseph</v>
       </c>
       <c r="L74" s="1">
         <f>VLOOKUP(J74,'Names with Seat Code'!A:F,6,FALSE)</f>
@@ -18550,14 +18549,14 @@
       </c>
       <c r="I75" s="1" t="str">
         <f>VLOOKUP(J75,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="J75">
         <v>62</v>
       </c>
       <c r="K75" t="str">
         <f>VLOOKUP(J75,'Names with Seat Code'!A:E,4,FALSE)</f>
-        <v>Joseph</v>
+        <v/>
       </c>
       <c r="L75" s="1" t="str">
         <f>VLOOKUP(J75,'Names with Seat Code'!A:F,6,FALSE)</f>
@@ -29638,7 +29637,7 @@
       </c>
       <c r="I52" s="6" t="str">
         <f>'Grad Raw Data'!H52</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="J52" s="6">
         <f>'Grad Raw Data'!G52</f>
@@ -30426,7 +30425,7 @@
       </c>
       <c r="H74" s="6" t="str">
         <f>'Grad Raw Data'!I74</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="I74" s="6" t="str">
         <f>'Grad Raw Data'!H74</f>
@@ -30462,7 +30461,7 @@
       </c>
       <c r="H75" s="6" t="str">
         <f>'Grad Raw Data'!I75</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="I75" s="6" t="str">
         <f>'Grad Raw Data'!H75</f>
@@ -39875,7 +39874,7 @@
       </c>
       <c r="C102" s="20" t="str">
         <f>'Grad Raw Data'!H52</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="D102" s="44" t="str">
         <f>'Grad Raw Data'!D52</f>
@@ -40835,11 +40834,11 @@
     <row r="146" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="20" t="str">
         <f>'Grad Raw Data'!I74</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="B146" s="20" t="str">
         <f>'Grad Raw Data'!K74</f>
-        <v/>
+        <v>Joseph</v>
       </c>
       <c r="C146" s="20" t="str">
         <f>'Grad Raw Data'!H74</f>
@@ -40879,11 +40878,11 @@
     <row r="148" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="20" t="str">
         <f>'Grad Raw Data'!I75</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="B148" s="20" t="str">
         <f>'Grad Raw Data'!K75</f>
-        <v>Joseph</v>
+        <v/>
       </c>
       <c r="C148" s="20" t="str">
         <f>'Grad Raw Data'!H75</f>
@@ -49101,7 +49100,7 @@
         <f>'Grad Raw Data'!I264</f>
         <v>Jiayu</v>
       </c>
-      <c r="B526" s="52"/>
+      <c r="B526" s="20"/>
       <c r="C526" s="20" t="str">
         <f>'Grad Raw Data'!H264</f>
         <v>Zheng</v>
@@ -49125,7 +49124,7 @@
     </row>
     <row r="528" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A528" s="51" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B528" s="50"/>
       <c r="C528" s="20"/>
@@ -50754,7 +50753,7 @@
       </c>
       <c r="C102" s="20" t="str">
         <f>'Grad Raw Data'!H52</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="D102" s="20"/>
       <c r="E102" s="20" t="str">
@@ -51428,11 +51427,11 @@
     <row r="146" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="20" t="str">
         <f>'Grad Raw Data'!I74</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="B146" s="20" t="str">
         <f>'Grad Raw Data'!K74</f>
-        <v/>
+        <v>Joseph</v>
       </c>
       <c r="C146" s="20" t="str">
         <f>'Grad Raw Data'!H74</f>
@@ -51459,11 +51458,11 @@
     <row r="148" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="20" t="str">
         <f>'Grad Raw Data'!I75</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="B148" s="20" t="str">
         <f>'Grad Raw Data'!K75</f>
-        <v>Joseph</v>
+        <v/>
       </c>
       <c r="C148" s="20" t="str">
         <f>'Grad Raw Data'!H75</f>
@@ -59074,7 +59073,7 @@
       </c>
       <c r="H40" s="31" t="str">
         <f>VLOOKUP(I40,'Names with Seat Code'!B:E,4)</f>
-        <v>Chite</v>
+        <v>Chute</v>
       </c>
       <c r="I40" s="25">
         <f>IF(B39+1&lt;DIRECTIONS!$E$24,B39+1,0)</f>
@@ -59774,7 +59773,7 @@
       </c>
       <c r="G62" s="31" t="str">
         <f>VLOOKUP(I62,'Names with Seat Code'!B:E,2)</f>
-        <v>Dante</v>
+        <v>Antonio</v>
       </c>
       <c r="H62" s="31" t="str">
         <f>VLOOKUP(I62,'Names with Seat Code'!B:E,4)</f>
@@ -59806,7 +59805,7 @@
       </c>
       <c r="G63" s="31" t="str">
         <f>VLOOKUP(I63,'Names with Seat Code'!B:E,2)</f>
-        <v>Antonio</v>
+        <v>Dante</v>
       </c>
       <c r="H63" s="31" t="str">
         <f>VLOOKUP(I63,'Names with Seat Code'!B:E,4)</f>

</xml_diff>

<commit_message>
wright and lee changes
</commit_message>
<xml_diff>
--- a/data/2026 GSMUD.xlsx
+++ b/data/2026 GSMUD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code Space\Git 2026 Grad\2026-Grad\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027EB726-55DC-47FB-B98A-5253AC41FE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E3E1FB-9521-4C51-A7A0-F9BF4044B672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DIRECTIONS" sheetId="9" r:id="rId1"/>
@@ -1105,9 +1105,6 @@
     <t>Jessica Wong</t>
   </si>
   <si>
-    <t>Jared Wright</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jamari Wright </t>
   </si>
   <si>
@@ -1517,6 +1514,9 @@
   </si>
   <si>
     <t>Will Chute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jared Wright </t>
   </si>
 </sst>
 </file>
@@ -2201,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="24" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -2209,7 +2209,7 @@
         <v>30</v>
       </c>
       <c r="O3" s="24" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2220,7 +2220,7 @@
         <v>31</v>
       </c>
       <c r="O4" s="24" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -2231,7 +2231,7 @@
         <v>32</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2239,7 +2239,7 @@
         <v>33</v>
       </c>
       <c r="O6" s="24" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -2247,7 +2247,7 @@
         <v>34</v>
       </c>
       <c r="O7" s="24" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -2258,7 +2258,7 @@
         <v>35</v>
       </c>
       <c r="O8" s="24" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2266,7 +2266,7 @@
         <v>36</v>
       </c>
       <c r="O9" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -2274,7 +2274,7 @@
         <v>37</v>
       </c>
       <c r="O10" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2282,7 +2282,7 @@
         <v>38</v>
       </c>
       <c r="O11" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -2290,7 +2290,7 @@
         <v>39</v>
       </c>
       <c r="O12" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -2304,7 +2304,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -2318,7 +2318,7 @@
         <v>41</v>
       </c>
       <c r="O14" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -2329,10 +2329,10 @@
         <v>10</v>
       </c>
       <c r="N15" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="O15" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -2343,10 +2343,10 @@
         <v>12</v>
       </c>
       <c r="N16" s="24" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O16" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -2357,10 +2357,10 @@
         <v>14</v>
       </c>
       <c r="N17" s="24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="O17" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -2371,7 +2371,7 @@
         <v>42</v>
       </c>
       <c r="O18" s="24" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -2448,7 +2448,7 @@
         <v>Abate</v>
       </c>
       <c r="F2" s="45" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -2500,7 +2500,7 @@
         <v>Abubakar</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2513,13 +2513,13 @@
         <v>Luis</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H5" t="s">
         <v>25</v>
@@ -2546,7 +2546,7 @@
         <v>Ahlert</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2567,7 +2567,7 @@
         <v>Aiello</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2609,7 +2609,7 @@
         <v>Amado</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2687,7 +2687,7 @@
         <v>Aquino</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2727,7 +2727,7 @@
         <v>Araujo</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2748,7 +2748,7 @@
         <v>Aretusi</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2826,7 +2826,7 @@
         <v>Batista</v>
       </c>
       <c r="F20" s="45" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2847,7 +2847,7 @@
         <v>Beaulieu</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2868,7 +2868,7 @@
         <v>Belfon</v>
       </c>
       <c r="F22" s="45" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2927,7 +2927,7 @@
         <v>Bhola</v>
       </c>
       <c r="F25" s="46" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2967,7 +2967,7 @@
         <v>Boucher</v>
       </c>
       <c r="F27" s="41" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3007,12 +3007,12 @@
         <v>Bowlin</v>
       </c>
       <c r="F29" s="41" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="45" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="40" t="str">
@@ -3199,7 +3199,7 @@
         <v>Carcione</v>
       </c>
       <c r="F39" s="41" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3261,7 +3261,7 @@
     </row>
     <row r="43" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="41" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B43" s="41"/>
       <c r="C43" s="40" t="str">
@@ -3315,7 +3315,7 @@
         <v>Cirrone</v>
       </c>
       <c r="F45" s="46" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3412,12 +3412,12 @@
         <v>Comenos</v>
       </c>
       <c r="F50" s="45" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="41" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B51" s="41"/>
       <c r="C51" s="40" t="str">
@@ -3611,7 +3611,7 @@
     </row>
     <row r="61" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B61" s="41"/>
       <c r="C61" s="40" t="str">
@@ -3639,10 +3639,10 @@
       </c>
       <c r="D62" s="40"/>
       <c r="E62" s="49" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F62" s="45" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3682,12 +3682,12 @@
         <v>Dean</v>
       </c>
       <c r="F64" s="45" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="41" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B65" s="41"/>
       <c r="C65" s="40" t="str">
@@ -3703,7 +3703,7 @@
         <v>Deji</v>
       </c>
       <c r="F65" s="41" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3743,7 +3743,7 @@
         <v>DiDonato</v>
       </c>
       <c r="F67" s="41" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3783,7 +3783,7 @@
         <v>DiSerio</v>
       </c>
       <c r="F69" s="41" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3804,7 +3804,7 @@
         <v>Donaghey</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3836,13 +3836,13 @@
         <v>Alana</v>
       </c>
       <c r="D72" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="E72" s="49" t="s">
         <v>469</v>
       </c>
-      <c r="E72" s="49" t="s">
-        <v>470</v>
-      </c>
       <c r="F72" s="46" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3882,7 +3882,7 @@
         <v>DuRoss</v>
       </c>
       <c r="F74" s="46" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3944,7 +3944,7 @@
     </row>
     <row r="78" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="45" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B78" s="41"/>
       <c r="C78" s="40" t="str">
@@ -3998,7 +3998,7 @@
         <v>Encarnacao</v>
       </c>
       <c r="F80" s="46" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4019,7 +4019,7 @@
         <v>Ewald</v>
       </c>
       <c r="F81" s="46" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4040,7 +4040,7 @@
         <v>Fantasia</v>
       </c>
       <c r="F82" s="45" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4121,7 +4121,7 @@
     </row>
     <row r="87" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="41" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B87" s="41"/>
       <c r="C87" s="40" t="str">
@@ -4175,7 +4175,7 @@
         <v>Forse</v>
       </c>
       <c r="F89" s="46" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4234,7 +4234,7 @@
         <v>Fucarile</v>
       </c>
       <c r="F92" s="45" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4293,7 +4293,7 @@
         <v>Gager</v>
       </c>
       <c r="F95" s="41" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4354,7 +4354,7 @@
         <v>Gauvin</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4489,7 +4489,7 @@
         <v>Gorski</v>
       </c>
       <c r="F105" s="41" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4510,7 +4510,7 @@
         <v>Gosdanian</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4588,7 +4588,7 @@
         <v>Hall</v>
       </c>
       <c r="F110" s="45" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4704,7 +4704,7 @@
         <v>Henri</v>
       </c>
       <c r="F116" s="46" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4763,7 +4763,7 @@
         <v>Hobson</v>
       </c>
       <c r="F119" s="41" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4803,7 +4803,7 @@
         <v>Houle</v>
       </c>
       <c r="F121" s="46" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4843,7 +4843,7 @@
         <v>Iosua</v>
       </c>
       <c r="F123" s="41" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5016,7 +5016,7 @@
         <v>Kaberle</v>
       </c>
       <c r="F132" s="46" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5037,7 +5037,7 @@
         <v>Kadric</v>
       </c>
       <c r="F133" s="46" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5058,7 +5058,7 @@
         <v>Keaveney</v>
       </c>
       <c r="F134" s="45" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5079,7 +5079,7 @@
         <v>Kenton</v>
       </c>
       <c r="F135" s="46" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5100,12 +5100,12 @@
         <v>Kiley</v>
       </c>
       <c r="F136" s="46" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A137" s="41" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B137" s="41"/>
       <c r="C137" s="40" t="str">
@@ -5159,17 +5159,17 @@
         <v>Lalicata</v>
       </c>
       <c r="F139" s="41" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A140" s="45" t="s">
-        <v>226</v>
+      <c r="A140" s="41" t="s">
+        <v>227</v>
       </c>
       <c r="B140" s="41"/>
       <c r="C140" s="40" t="str">
         <f t="shared" si="9"/>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="D140" s="40" t="str">
         <f t="shared" si="10"/>
@@ -5179,18 +5179,15 @@
         <f t="shared" si="11"/>
         <v>Laurino</v>
       </c>
-      <c r="F140" s="45" t="s">
-        <v>393</v>
-      </c>
     </row>
     <row r="141" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A141" s="41" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B141" s="41"/>
       <c r="C141" s="40" t="str">
         <f t="shared" si="9"/>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="D141" s="40" t="str">
         <f t="shared" si="10"/>
@@ -5200,7 +5197,9 @@
         <f t="shared" si="11"/>
         <v>Laurino</v>
       </c>
-      <c r="F141" s="41"/>
+      <c r="F141" s="45" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="142" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A142" s="45" t="s">
@@ -5220,21 +5219,21 @@
         <v>Layne</v>
       </c>
       <c r="F142" s="45" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="41" t="s">
-        <v>229</v>
+      <c r="A143" s="45" t="s">
+        <v>230</v>
       </c>
       <c r="B143" s="41"/>
       <c r="C143" s="40" t="str">
         <f t="shared" si="9"/>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="D143" s="40" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>James</v>
       </c>
       <c r="E143" s="40" t="str">
         <f t="shared" si="11"/>
@@ -5244,16 +5243,16 @@
     </row>
     <row r="144" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A144" s="45" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B144" s="41"/>
       <c r="C144" s="40" t="str">
         <f t="shared" si="9"/>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="D144" s="40" t="str">
         <f t="shared" si="10"/>
-        <v>James</v>
+        <v/>
       </c>
       <c r="E144" s="40" t="str">
         <f t="shared" si="11"/>
@@ -5355,7 +5354,7 @@
         <v>Lizotte</v>
       </c>
       <c r="F149" s="46" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5376,7 +5375,7 @@
         <v>Lusk</v>
       </c>
       <c r="F150" s="46" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="151" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5416,7 +5415,7 @@
         <v>Maganzini</v>
       </c>
       <c r="F152" s="45" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="153" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5475,7 +5474,7 @@
         <v>Maness</v>
       </c>
       <c r="F155" s="41" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5579,7 +5578,7 @@
     </row>
     <row r="161" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A161" s="47" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B161" s="41"/>
       <c r="C161" s="40" t="str">
@@ -5598,7 +5597,7 @@
     </row>
     <row r="162" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A162" s="48" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B162" s="41"/>
       <c r="C162" s="40" t="str">
@@ -5709,7 +5708,7 @@
         <v>McLaughlin-Shostak</v>
       </c>
       <c r="F167" s="41" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5730,7 +5729,7 @@
         <v>McMenimen</v>
       </c>
       <c r="F168" s="45" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5808,7 +5807,7 @@
         <v>Miceli</v>
       </c>
       <c r="F172" s="46" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="173" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5832,7 +5831,7 @@
     </row>
     <row r="174" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A174" s="48" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B174" s="41"/>
       <c r="C174" s="40" t="str">
@@ -5867,7 +5866,7 @@
         <v>Moller</v>
       </c>
       <c r="F175" s="41" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5888,7 +5887,7 @@
         <v>Moreira</v>
       </c>
       <c r="F176" s="45" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5966,7 +5965,7 @@
         <v>Muller</v>
       </c>
       <c r="F180" s="45" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6065,7 +6064,7 @@
         <v>Nguyen</v>
       </c>
       <c r="F185" s="41" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="186" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6105,7 +6104,7 @@
         <v>Norris</v>
       </c>
       <c r="F187" s="41" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="188" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6145,7 +6144,7 @@
         <v>Ortins</v>
       </c>
       <c r="F189" s="41" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="190" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6206,7 +6205,7 @@
         <v>Patel</v>
       </c>
       <c r="F192" s="46" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6246,7 +6245,7 @@
         <v>Petrin</v>
       </c>
       <c r="F194" s="45" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="195" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6270,7 +6269,7 @@
     </row>
     <row r="196" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A196" s="48" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B196" s="41"/>
       <c r="C196" s="40" t="str">
@@ -6305,7 +6304,7 @@
         <v>Pomerantz</v>
       </c>
       <c r="F197" s="46" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="198" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6326,12 +6325,12 @@
         <v>Poudyal</v>
       </c>
       <c r="F198" s="45" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="199" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A199" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B199" s="41"/>
       <c r="C199" s="40" t="str">
@@ -6368,7 +6367,7 @@
         <v>Rai</v>
       </c>
       <c r="F200" s="46" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="201" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6446,7 +6445,7 @@
         <v>Richter</v>
       </c>
       <c r="F204" s="46" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="205" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6467,7 +6466,7 @@
         <v>Robichaud</v>
       </c>
       <c r="F205" s="46" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="206" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6583,7 +6582,7 @@
         <v>Rojas</v>
       </c>
       <c r="F211" s="41" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="212" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6607,7 +6606,7 @@
     </row>
     <row r="213" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A213" s="41" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B213" s="41"/>
       <c r="C213" s="40" t="str">
@@ -6644,7 +6643,7 @@
         <v>Sardinha</v>
       </c>
       <c r="F214" s="45" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="215" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6665,7 +6664,7 @@
         <v>Sarre</v>
       </c>
       <c r="F215" s="41" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="216" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6724,7 +6723,7 @@
         <v>Schrager</v>
       </c>
       <c r="F218" s="45" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="219" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6783,12 +6782,12 @@
         <v>Selvakumar</v>
       </c>
       <c r="F221" s="46" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="222" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A222" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B222" s="41"/>
       <c r="C222" s="40" t="str">
@@ -6842,7 +6841,7 @@
         <v>Shediac</v>
       </c>
       <c r="F224" s="45" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="225" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6882,7 +6881,7 @@
         <v>Siciliano</v>
       </c>
       <c r="F226" s="45" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="227" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6922,7 +6921,7 @@
         <v>Skenderian</v>
       </c>
       <c r="F228" s="46" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="229" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7002,7 +7001,7 @@
         <v>Soto</v>
       </c>
       <c r="F232" s="45" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="233" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7080,7 +7079,7 @@
         <v>Staffier</v>
       </c>
       <c r="F236" s="46" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="237" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7101,7 +7100,7 @@
         <v>Stathoulopoulos</v>
       </c>
       <c r="F237" s="46" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="238" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7200,7 +7199,7 @@
         <v>Taubman</v>
       </c>
       <c r="F242" s="45" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="243" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7221,7 +7220,7 @@
         <v>Tawadros</v>
       </c>
       <c r="F243" s="41" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="244" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7282,7 +7281,7 @@
         <v>Travassos</v>
       </c>
       <c r="F246" s="45" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="247" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7303,7 +7302,7 @@
         <v>Upton</v>
       </c>
       <c r="F247" s="46" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="248" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7336,7 +7335,7 @@
       </c>
       <c r="D249" s="40"/>
       <c r="E249" s="49" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F249" s="41"/>
     </row>
@@ -7350,10 +7349,10 @@
         <v>Katherine</v>
       </c>
       <c r="D250" s="49" t="s">
+        <v>466</v>
+      </c>
+      <c r="E250" s="49" t="s">
         <v>467</v>
-      </c>
-      <c r="E250" s="49" t="s">
-        <v>468</v>
       </c>
       <c r="F250" s="45"/>
     </row>
@@ -7394,7 +7393,7 @@
         <v>Viliott</v>
       </c>
       <c r="F252" s="45" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="253" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7415,7 +7414,7 @@
         <v>Vitarisi</v>
       </c>
       <c r="F253" s="46" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="254" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7591,7 +7590,7 @@
     </row>
     <row r="263" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A263" s="41" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B263" s="41"/>
       <c r="C263" s="40" t="str">
@@ -7607,7 +7606,7 @@
         <v>Williams</v>
       </c>
       <c r="F263" s="41" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="264" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7630,44 +7629,44 @@
       <c r="F264" s="45"/>
     </row>
     <row r="265" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A265" s="41" t="s">
+      <c r="A265" s="45" t="s">
         <v>344</v>
       </c>
       <c r="C265" s="40" t="str">
-        <f t="shared" si="15"/>
-        <v>Jared</v>
+        <f>IF(ISERROR( FIND(",",TRIM(A265))),LEFT(TRIM(A265), FIND(" ",TRIM(A265))-1),MID(TRIM(A265),LEN(C265)+3,FIND(" ",TRIM(A265)&amp;" ",LEN(C265)+3)-LEN(C265)-2))</f>
+        <v>Jamari</v>
       </c>
       <c r="D265" s="40" t="str">
-        <f t="shared" si="16"/>
+        <f>IF(ISERROR(FIND(",",TRIM(A265))),IF(LEN(TRIM(A265))-LEN(SUBSTITUTE(TRIM(A265)," ",""))=2,MID(TRIM(A265),LEN(C265)+2,FIND(" ",TRIM(A265),LEN(C265)+2)-LEN(C265)-2),""),MID(TRIM(A265),3+LEN(C265)+LEN(E265),30))</f>
         <v/>
       </c>
       <c r="E265" s="40" t="str">
-        <f t="shared" si="17"/>
+        <f>IF(ISERROR(FIND(",",TRIM(A265))),MID(TRIM(A265),1+LEN(TRIM(A265))-LEN(SUBSTITUTE(TRIM(A265)," ",""))+LEN(C265)+LEN(D265),30),LEFT(TRIM(A265), FIND(",",TRIM(A265))-1))</f>
         <v>Wright</v>
       </c>
       <c r="F265" s="41"/>
     </row>
     <row r="266" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A266" s="45" t="s">
-        <v>345</v>
+        <v>481</v>
       </c>
       <c r="C266" s="40" t="str">
-        <f t="shared" si="15"/>
-        <v>Jamari</v>
+        <f>IF(ISERROR( FIND(",",TRIM(A266))),LEFT(TRIM(A266), FIND(" ",TRIM(A266))-1),MID(TRIM(A266),LEN(C266)+3,FIND(" ",TRIM(A266)&amp;" ",LEN(C266)+3)-LEN(C266)-2))</f>
+        <v>Jared</v>
       </c>
       <c r="D266" s="40" t="str">
-        <f t="shared" si="16"/>
+        <f>IF(ISERROR(FIND(",",TRIM(A266))),IF(LEN(TRIM(A266))-LEN(SUBSTITUTE(TRIM(A266)," ",""))=2,MID(TRIM(A266),LEN(C266)+2,FIND(" ",TRIM(A266),LEN(C266)+2)-LEN(C266)-2),""),MID(TRIM(A266),3+LEN(C266)+LEN(E266),30))</f>
         <v/>
       </c>
       <c r="E266" s="40" t="str">
-        <f t="shared" si="17"/>
+        <f>IF(ISERROR(FIND(",",TRIM(A266))),MID(TRIM(A266),1+LEN(TRIM(A266))-LEN(SUBSTITUTE(TRIM(A266)," ",""))+LEN(C266)+LEN(D266),30),LEFT(TRIM(A266), FIND(",",TRIM(A266))-1))</f>
         <v>Wright</v>
       </c>
       <c r="F266" s="45"/>
     </row>
     <row r="267" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A267" s="41" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C267" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7685,7 +7684,7 @@
     </row>
     <row r="268" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A268" s="45" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C268" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7700,12 +7699,12 @@
         <v>Zani</v>
       </c>
       <c r="F268" s="45" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="269" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A269" s="41" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C269" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7720,7 +7719,7 @@
         <v>Zheng</v>
       </c>
       <c r="F269" s="41" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.2">
@@ -7797,7 +7796,7 @@
       <c r="H2" s="42"/>
       <c r="I2" s="42"/>
       <c r="L2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -7828,7 +7827,7 @@
       <c r="H3" s="42"/>
       <c r="I3" s="42"/>
       <c r="L3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -7859,7 +7858,7 @@
       <c r="H4" s="42"/>
       <c r="I4" s="42"/>
       <c r="L4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -7890,7 +7889,7 @@
       <c r="H5" s="42"/>
       <c r="I5" s="42"/>
       <c r="L5" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -7949,7 +7948,7 @@
       <c r="H7" s="42"/>
       <c r="I7" s="42"/>
       <c r="L7" s="22" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -7983,7 +7982,7 @@
         <v>30</v>
       </c>
       <c r="M8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -8017,7 +8016,7 @@
         <v>87</v>
       </c>
       <c r="M9" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -8051,7 +8050,7 @@
         <v>31</v>
       </c>
       <c r="M10" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -8085,7 +8084,7 @@
         <v>32</v>
       </c>
       <c r="M11" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -8119,7 +8118,7 @@
         <v>33</v>
       </c>
       <c r="M12" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -8153,7 +8152,7 @@
         <v>34</v>
       </c>
       <c r="M13" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -8187,7 +8186,7 @@
         <v>35</v>
       </c>
       <c r="M14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -8221,7 +8220,7 @@
         <v>36</v>
       </c>
       <c r="M15" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -8255,7 +8254,7 @@
         <v>37</v>
       </c>
       <c r="M16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -8289,7 +8288,7 @@
         <v>38</v>
       </c>
       <c r="M17" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -8323,7 +8322,7 @@
         <v>39</v>
       </c>
       <c r="M18" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -8357,7 +8356,7 @@
         <v>40</v>
       </c>
       <c r="M19" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -8391,7 +8390,7 @@
         <v>41</v>
       </c>
       <c r="M20" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -8422,10 +8421,10 @@
       <c r="H21" s="42"/>
       <c r="I21" s="42"/>
       <c r="L21" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="M21" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -8456,10 +8455,10 @@
       <c r="H22" s="42"/>
       <c r="I22" s="42"/>
       <c r="L22" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M22" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -8490,10 +8489,10 @@
       <c r="H23" s="42"/>
       <c r="I23" s="42"/>
       <c r="L23" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="M23" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -8527,7 +8526,7 @@
         <v>42</v>
       </c>
       <c r="M24" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -10098,7 +10097,7 @@
         <v/>
       </c>
       <c r="E81" s="39" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F81" s="39" t="str">
         <f>'Raw Name Splitter'!F81</f>
@@ -11734,7 +11733,7 @@
       </c>
       <c r="C140" s="39" t="str">
         <f>'Raw Name Splitter'!C140</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="D140" s="39" t="str">
         <f>'Raw Name Splitter'!D140</f>
@@ -11745,7 +11744,7 @@
         <v>Laurino</v>
       </c>
       <c r="F140" s="39" t="str">
-        <f>'Raw Name Splitter'!F140</f>
+        <f>'Raw Name Splitter'!F141</f>
         <v>Matthew La-Ree-No</v>
       </c>
       <c r="H140" s="42"/>
@@ -11762,7 +11761,7 @@
       </c>
       <c r="C141" s="39" t="str">
         <f>'Raw Name Splitter'!C141</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="D141" s="39" t="str">
         <f>'Raw Name Splitter'!D141</f>
@@ -11772,9 +11771,9 @@
         <f>'Raw Name Splitter'!E141</f>
         <v>Laurino</v>
       </c>
-      <c r="F141" s="39">
-        <f>'Raw Name Splitter'!F141</f>
-        <v>0</v>
+      <c r="F141" s="39" t="e">
+        <f>'Raw Name Splitter'!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="H141" s="42"/>
       <c r="I141" s="42"/>
@@ -11818,11 +11817,11 @@
       </c>
       <c r="C143" s="39" t="str">
         <f>'Raw Name Splitter'!C143</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="D143" s="39" t="str">
         <f>'Raw Name Splitter'!D143</f>
-        <v/>
+        <v>James</v>
       </c>
       <c r="E143" s="39" t="str">
         <f>'Raw Name Splitter'!E143</f>
@@ -11846,11 +11845,11 @@
       </c>
       <c r="C144" s="39" t="str">
         <f>'Raw Name Splitter'!C144</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="D144" s="39" t="str">
         <f>'Raw Name Splitter'!D144</f>
-        <v>James</v>
+        <v/>
       </c>
       <c r="E144" s="39" t="str">
         <f>'Raw Name Splitter'!E144</f>
@@ -14771,7 +14770,7 @@
         <v>Colby</v>
       </c>
       <c r="E249" s="39" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F249" s="39">
         <f>'Raw Name Splitter'!F249</f>
@@ -15205,7 +15204,7 @@
       </c>
       <c r="C265" s="39" t="str">
         <f>'Raw Name Splitter'!C265</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="D265" s="39" t="str">
         <f>'Raw Name Splitter'!D265</f>
@@ -15233,7 +15232,7 @@
       </c>
       <c r="C266" s="39" t="str">
         <f>'Raw Name Splitter'!C266</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="D266" s="39" t="str">
         <f>'Raw Name Splitter'!D266</f>
@@ -15334,13 +15333,13 @@
         <v>87</v>
       </c>
       <c r="C270" s="39" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E270" s="39" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F270" s="39" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -21426,7 +21425,7 @@
       </c>
       <c r="I141" s="1" t="str">
         <f>VLOOKUP(J141,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="J141">
         <v>128</v>
@@ -21470,7 +21469,7 @@
       </c>
       <c r="I142" s="1" t="str">
         <f>VLOOKUP(J142,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="J142">
         <v>129</v>
@@ -21479,9 +21478,9 @@
         <f>VLOOKUP(J142,'Names with Seat Code'!A:E,4,FALSE)</f>
         <v/>
       </c>
-      <c r="L142" s="1">
+      <c r="L142" s="1" t="e">
         <f>VLOOKUP(J142,'Names with Seat Code'!A:F,6,FALSE)</f>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
@@ -21558,14 +21557,14 @@
       </c>
       <c r="I144" s="1" t="str">
         <f>VLOOKUP(J144,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="J144">
         <v>131</v>
       </c>
       <c r="K144" t="str">
         <f>VLOOKUP(J144,'Names with Seat Code'!A:E,4,FALSE)</f>
-        <v/>
+        <v>James</v>
       </c>
       <c r="L144" s="1">
         <f>VLOOKUP(J144,'Names with Seat Code'!A:F,6,FALSE)</f>
@@ -21602,14 +21601,14 @@
       </c>
       <c r="I145" s="1" t="str">
         <f>VLOOKUP(J145,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="J145">
         <v>132</v>
       </c>
       <c r="K145" t="str">
         <f>VLOOKUP(J145,'Names with Seat Code'!A:E,4,FALSE)</f>
-        <v>James</v>
+        <v/>
       </c>
       <c r="L145" s="1">
         <f>VLOOKUP(J145,'Names with Seat Code'!A:F,6,FALSE)</f>
@@ -26662,7 +26661,7 @@
       </c>
       <c r="I260" s="1" t="str">
         <f>VLOOKUP(J260,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="J260">
         <v>242</v>
@@ -26680,7 +26679,7 @@
         <v>68</v>
       </c>
       <c r="C261" s="6">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D261" s="7" t="s">
         <v>53</v>
@@ -26702,7 +26701,7 @@
       </c>
       <c r="I261" s="1" t="str">
         <f>VLOOKUP(J261,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="J261">
         <v>243</v>
@@ -26720,7 +26719,7 @@
         <v>68</v>
       </c>
       <c r="C262" s="6">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D262" s="7" t="s">
         <v>53</v>
@@ -26760,7 +26759,7 @@
         <v>68</v>
       </c>
       <c r="C263" s="6">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D263" s="7" t="s">
         <v>53</v>
@@ -26800,7 +26799,7 @@
         <v>68</v>
       </c>
       <c r="C264" s="6">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D264" s="7" t="s">
         <v>53</v>
@@ -32876,7 +32875,7 @@
       </c>
       <c r="H141" s="6" t="str">
         <f>'Grad Raw Data'!I141</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="I141" s="6" t="str">
         <f>'Grad Raw Data'!H141</f>
@@ -32913,7 +32912,7 @@
       </c>
       <c r="H142" s="6" t="str">
         <f>'Grad Raw Data'!I142</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="I142" s="6" t="str">
         <f>'Grad Raw Data'!H142</f>
@@ -32987,7 +32986,7 @@
       </c>
       <c r="H144" s="6" t="str">
         <f>'Grad Raw Data'!I144</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="I144" s="6" t="str">
         <f>'Grad Raw Data'!H144</f>
@@ -33024,7 +33023,7 @@
       </c>
       <c r="H145" s="6" t="str">
         <f>'Grad Raw Data'!I145</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="I145" s="6" t="str">
         <f>'Grad Raw Data'!H145</f>
@@ -37275,7 +37274,7 @@
       </c>
       <c r="H260" s="6" t="str">
         <f>'Grad Raw Data'!I260</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="I260" s="6" t="str">
         <f>'Grad Raw Data'!H260</f>
@@ -37310,7 +37309,7 @@
       </c>
       <c r="H261" s="6" t="str">
         <f>'Grad Raw Data'!I261</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="I261" s="6" t="str">
         <f>'Grad Raw Data'!H261</f>
@@ -43782,7 +43781,7 @@
     <row r="280" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A280" s="20" t="str">
         <f>'Grad Raw Data'!I141</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="B280" s="20" t="str">
         <f>'Grad Raw Data'!K141</f>
@@ -43826,7 +43825,7 @@
     <row r="282" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A282" s="20" t="str">
         <f>'Grad Raw Data'!I142</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="B282" s="20" t="str">
         <f>'Grad Raw Data'!K142</f>
@@ -43853,9 +43852,9 @@
       </c>
     </row>
     <row r="283" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A283" s="16">
+      <c r="A283" s="16" t="e">
         <f>'Grad Raw Data'!L142</f>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
       <c r="B283" s="20"/>
       <c r="C283" s="20"/>
@@ -43914,11 +43913,11 @@
     <row r="286" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A286" s="20" t="str">
         <f>'Grad Raw Data'!I144</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="B286" s="20" t="str">
         <f>'Grad Raw Data'!K144</f>
-        <v/>
+        <v>James</v>
       </c>
       <c r="C286" s="20" t="str">
         <f>'Grad Raw Data'!H144</f>
@@ -43958,11 +43957,11 @@
     <row r="288" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A288" s="20" t="str">
         <f>'Grad Raw Data'!I145</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="B288" s="20" t="str">
         <f>'Grad Raw Data'!K145</f>
-        <v>James</v>
+        <v/>
       </c>
       <c r="C288" s="20" t="str">
         <f>'Grad Raw Data'!H145</f>
@@ -48990,7 +48989,7 @@
     <row r="518" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A518" s="20" t="str">
         <f>'Grad Raw Data'!I260</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="B518" s="20"/>
       <c r="C518" s="20" t="str">
@@ -49017,7 +49016,7 @@
     <row r="520" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A520" s="20" t="str">
         <f>'Grad Raw Data'!I261</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="B520" s="50"/>
       <c r="C520" s="20" t="str">
@@ -49124,7 +49123,7 @@
     </row>
     <row r="528" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A528" s="51" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B528" s="50"/>
       <c r="C528" s="20"/>
@@ -53504,7 +53503,7 @@
     <row r="280" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A280" s="20" t="str">
         <f>'Grad Raw Data'!I141</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="B280" s="20" t="str">
         <f>'Grad Raw Data'!K141</f>
@@ -53535,7 +53534,7 @@
     <row r="282" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A282" s="20" t="str">
         <f>'Grad Raw Data'!I142</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="B282" s="20" t="str">
         <f>'Grad Raw Data'!K142</f>
@@ -53597,11 +53596,11 @@
     <row r="286" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A286" s="20" t="str">
         <f>'Grad Raw Data'!I144</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="B286" s="20" t="str">
         <f>'Grad Raw Data'!K144</f>
-        <v/>
+        <v>James</v>
       </c>
       <c r="C286" s="20" t="str">
         <f>'Grad Raw Data'!H144</f>
@@ -53628,11 +53627,11 @@
     <row r="288" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A288" s="20" t="str">
         <f>'Grad Raw Data'!I145</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="B288" s="20" t="str">
         <f>'Grad Raw Data'!K145</f>
-        <v>James</v>
+        <v/>
       </c>
       <c r="C288" s="20" t="str">
         <f>'Grad Raw Data'!H145</f>
@@ -57193,7 +57192,7 @@
     <row r="518" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A518" s="20" t="str">
         <f>'Grad Raw Data'!I260</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="B518" s="20" t="str">
         <f>'Grad Raw Data'!K259</f>
@@ -57224,7 +57223,7 @@
     <row r="520" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A520" s="20" t="str">
         <f>'Grad Raw Data'!I261</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="B520" s="20"/>
       <c r="C520" s="20" t="str">
@@ -61917,7 +61916,7 @@
       </c>
       <c r="G129" s="31" t="str">
         <f>VLOOKUP(I129,'Names with Seat Code'!B:E,2)</f>
-        <v>Matthew</v>
+        <v>Jonathan</v>
       </c>
       <c r="H129" s="31" t="str">
         <f>VLOOKUP(I129,'Names with Seat Code'!B:E,4)</f>
@@ -61949,7 +61948,7 @@
       </c>
       <c r="G130" s="31" t="str">
         <f>VLOOKUP(I130,'Names with Seat Code'!B:E,2)</f>
-        <v>Jonathan</v>
+        <v>Matthew</v>
       </c>
       <c r="H130" s="31" t="str">
         <f>VLOOKUP(I130,'Names with Seat Code'!B:E,4)</f>
@@ -62013,7 +62012,7 @@
       </c>
       <c r="G132" s="31" t="str">
         <f>VLOOKUP(I132,'Names with Seat Code'!B:E,2)</f>
-        <v>Jonathan</v>
+        <v>Austin</v>
       </c>
       <c r="H132" s="31" t="str">
         <f>VLOOKUP(I132,'Names with Seat Code'!B:E,4)</f>
@@ -64765,7 +64764,7 @@
       </c>
       <c r="G218" s="31" t="str">
         <f>VLOOKUP(I218,'Names with Seat Code'!B:E,2)</f>
-        <v>Austin</v>
+        <v>Jonathan</v>
       </c>
       <c r="H218" s="31" t="str">
         <f>VLOOKUP(I218,'Names with Seat Code'!B:E,4)</f>
@@ -68285,7 +68284,7 @@
       </c>
       <c r="G328" s="31" t="str">
         <f>VLOOKUP(I328,'Names with Seat Code'!B:E,2)</f>
-        <v>Jared</v>
+        <v>Jamari</v>
       </c>
       <c r="H328" s="31" t="str">
         <f>VLOOKUP(I328,'Names with Seat Code'!B:E,4)</f>
@@ -68317,7 +68316,7 @@
       </c>
       <c r="G329" s="31" t="str">
         <f>VLOOKUP(I329,'Names with Seat Code'!B:E,2)</f>
-        <v>Jamari</v>
+        <v>Jared</v>
       </c>
       <c r="H329" s="31" t="str">
         <f>VLOOKUP(I329,'Names with Seat Code'!B:E,4)</f>

</xml_diff>

<commit_message>
FINAL EDITION fixed Lee, Weaver, last row print
</commit_message>
<xml_diff>
--- a/data/2026 GSMUD.xlsx
+++ b/data/2026 GSMUD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code Space\Git 2026 Grad\2026-Grad\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E3E1FB-9521-4C51-A7A0-F9BF4044B672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E145ABA0-5420-4FB3-B4B2-73A9BE6FDF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DIRECTIONS" sheetId="9" r:id="rId1"/>
@@ -1084,9 +1084,6 @@
     <t>Jacob Michael Ward</t>
   </si>
   <si>
-    <t xml:space="preserve">Tess  Weaver </t>
-  </si>
-  <si>
     <t>Kyle Weaver</t>
   </si>
   <si>
@@ -1517,6 +1514,9 @@
   </si>
   <si>
     <t xml:space="preserve">Jared Wright </t>
+  </si>
+  <si>
+    <t>Tess Weaver</t>
   </si>
 </sst>
 </file>
@@ -2201,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="N2" s="24" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -2209,7 +2209,7 @@
         <v>30</v>
       </c>
       <c r="O3" s="24" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2220,7 +2220,7 @@
         <v>31</v>
       </c>
       <c r="O4" s="24" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -2231,7 +2231,7 @@
         <v>32</v>
       </c>
       <c r="O5" s="24" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2239,7 +2239,7 @@
         <v>33</v>
       </c>
       <c r="O6" s="24" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -2247,7 +2247,7 @@
         <v>34</v>
       </c>
       <c r="O7" s="24" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -2258,7 +2258,7 @@
         <v>35</v>
       </c>
       <c r="O8" s="24" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2266,7 +2266,7 @@
         <v>36</v>
       </c>
       <c r="O9" s="24" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -2274,7 +2274,7 @@
         <v>37</v>
       </c>
       <c r="O10" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2282,7 +2282,7 @@
         <v>38</v>
       </c>
       <c r="O11" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -2290,7 +2290,7 @@
         <v>39</v>
       </c>
       <c r="O12" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -2304,7 +2304,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -2318,7 +2318,7 @@
         <v>41</v>
       </c>
       <c r="O14" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -2329,10 +2329,10 @@
         <v>10</v>
       </c>
       <c r="N15" s="24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="O15" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -2343,10 +2343,10 @@
         <v>12</v>
       </c>
       <c r="N16" s="24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="O16" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -2357,10 +2357,10 @@
         <v>14</v>
       </c>
       <c r="N17" s="24" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O17" s="24" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -2371,7 +2371,7 @@
         <v>42</v>
       </c>
       <c r="O18" s="24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -2448,7 +2448,7 @@
         <v>Abate</v>
       </c>
       <c r="F2" s="45" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -2500,7 +2500,7 @@
         <v>Abubakar</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2513,13 +2513,13 @@
         <v>Luis</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H5" t="s">
         <v>25</v>
@@ -2546,7 +2546,7 @@
         <v>Ahlert</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2567,7 +2567,7 @@
         <v>Aiello</v>
       </c>
       <c r="F7" s="41" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2609,7 +2609,7 @@
         <v>Amado</v>
       </c>
       <c r="F9" s="41" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2687,7 +2687,7 @@
         <v>Aquino</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2727,7 +2727,7 @@
         <v>Araujo</v>
       </c>
       <c r="F15" s="41" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -2748,7 +2748,7 @@
         <v>Aretusi</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2826,7 +2826,7 @@
         <v>Batista</v>
       </c>
       <c r="F20" s="45" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2847,7 +2847,7 @@
         <v>Beaulieu</v>
       </c>
       <c r="F21" s="41" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2868,7 +2868,7 @@
         <v>Belfon</v>
       </c>
       <c r="F22" s="45" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2927,7 +2927,7 @@
         <v>Bhola</v>
       </c>
       <c r="F25" s="46" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2967,7 +2967,7 @@
         <v>Boucher</v>
       </c>
       <c r="F27" s="41" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3007,12 +3007,12 @@
         <v>Bowlin</v>
       </c>
       <c r="F29" s="41" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="45" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="40" t="str">
@@ -3199,7 +3199,7 @@
         <v>Carcione</v>
       </c>
       <c r="F39" s="41" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3261,7 +3261,7 @@
     </row>
     <row r="43" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="41" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B43" s="41"/>
       <c r="C43" s="40" t="str">
@@ -3315,7 +3315,7 @@
         <v>Cirrone</v>
       </c>
       <c r="F45" s="46" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3412,12 +3412,12 @@
         <v>Comenos</v>
       </c>
       <c r="F50" s="45" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="41" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B51" s="41"/>
       <c r="C51" s="40" t="str">
@@ -3611,7 +3611,7 @@
     </row>
     <row r="61" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B61" s="41"/>
       <c r="C61" s="40" t="str">
@@ -3639,10 +3639,10 @@
       </c>
       <c r="D62" s="40"/>
       <c r="E62" s="49" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F62" s="45" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3682,12 +3682,12 @@
         <v>Dean</v>
       </c>
       <c r="F64" s="45" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="41" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B65" s="41"/>
       <c r="C65" s="40" t="str">
@@ -3703,7 +3703,7 @@
         <v>Deji</v>
       </c>
       <c r="F65" s="41" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3743,7 +3743,7 @@
         <v>DiDonato</v>
       </c>
       <c r="F67" s="41" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3783,7 +3783,7 @@
         <v>DiSerio</v>
       </c>
       <c r="F69" s="41" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3804,7 +3804,7 @@
         <v>Donaghey</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3836,13 +3836,13 @@
         <v>Alana</v>
       </c>
       <c r="D72" s="49" t="s">
+        <v>467</v>
+      </c>
+      <c r="E72" s="49" t="s">
         <v>468</v>
       </c>
-      <c r="E72" s="49" t="s">
-        <v>469</v>
-      </c>
       <c r="F72" s="46" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3882,7 +3882,7 @@
         <v>DuRoss</v>
       </c>
       <c r="F74" s="46" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -3944,7 +3944,7 @@
     </row>
     <row r="78" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="45" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B78" s="41"/>
       <c r="C78" s="40" t="str">
@@ -3998,7 +3998,7 @@
         <v>Encarnacao</v>
       </c>
       <c r="F80" s="46" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4019,7 +4019,7 @@
         <v>Ewald</v>
       </c>
       <c r="F81" s="46" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4040,7 +4040,7 @@
         <v>Fantasia</v>
       </c>
       <c r="F82" s="45" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4121,7 +4121,7 @@
     </row>
     <row r="87" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="41" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B87" s="41"/>
       <c r="C87" s="40" t="str">
@@ -4175,7 +4175,7 @@
         <v>Forse</v>
       </c>
       <c r="F89" s="46" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4234,7 +4234,7 @@
         <v>Fucarile</v>
       </c>
       <c r="F92" s="45" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4293,7 +4293,7 @@
         <v>Gager</v>
       </c>
       <c r="F95" s="41" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4354,7 +4354,7 @@
         <v>Gauvin</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4489,7 +4489,7 @@
         <v>Gorski</v>
       </c>
       <c r="F105" s="41" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4510,7 +4510,7 @@
         <v>Gosdanian</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4588,7 +4588,7 @@
         <v>Hall</v>
       </c>
       <c r="F110" s="45" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4704,7 +4704,7 @@
         <v>Henri</v>
       </c>
       <c r="F116" s="46" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4763,7 +4763,7 @@
         <v>Hobson</v>
       </c>
       <c r="F119" s="41" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4803,7 +4803,7 @@
         <v>Houle</v>
       </c>
       <c r="F121" s="46" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -4843,7 +4843,7 @@
         <v>Iosua</v>
       </c>
       <c r="F123" s="41" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5016,7 +5016,7 @@
         <v>Kaberle</v>
       </c>
       <c r="F132" s="46" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5037,7 +5037,7 @@
         <v>Kadric</v>
       </c>
       <c r="F133" s="46" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5058,7 +5058,7 @@
         <v>Keaveney</v>
       </c>
       <c r="F134" s="45" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5079,7 +5079,7 @@
         <v>Kenton</v>
       </c>
       <c r="F135" s="46" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5100,12 +5100,12 @@
         <v>Kiley</v>
       </c>
       <c r="F136" s="46" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A137" s="41" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B137" s="41"/>
       <c r="C137" s="40" t="str">
@@ -5159,7 +5159,7 @@
         <v>Lalicata</v>
       </c>
       <c r="F139" s="41" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5198,7 +5198,7 @@
         <v>Laurino</v>
       </c>
       <c r="F141" s="45" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5219,7 +5219,7 @@
         <v>Layne</v>
       </c>
       <c r="F142" s="45" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5354,7 +5354,7 @@
         <v>Lizotte</v>
       </c>
       <c r="F149" s="46" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5375,7 +5375,7 @@
         <v>Lusk</v>
       </c>
       <c r="F150" s="46" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="151" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5415,7 +5415,7 @@
         <v>Maganzini</v>
       </c>
       <c r="F152" s="45" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="153" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5474,7 +5474,7 @@
         <v>Maness</v>
       </c>
       <c r="F155" s="41" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5578,7 +5578,7 @@
     </row>
     <row r="161" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A161" s="47" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B161" s="41"/>
       <c r="C161" s="40" t="str">
@@ -5597,7 +5597,7 @@
     </row>
     <row r="162" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A162" s="48" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B162" s="41"/>
       <c r="C162" s="40" t="str">
@@ -5708,7 +5708,7 @@
         <v>McLaughlin-Shostak</v>
       </c>
       <c r="F167" s="41" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5729,7 +5729,7 @@
         <v>McMenimen</v>
       </c>
       <c r="F168" s="45" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5807,7 +5807,7 @@
         <v>Miceli</v>
       </c>
       <c r="F172" s="46" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="173" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5831,7 +5831,7 @@
     </row>
     <row r="174" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A174" s="48" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B174" s="41"/>
       <c r="C174" s="40" t="str">
@@ -5866,7 +5866,7 @@
         <v>Moller</v>
       </c>
       <c r="F175" s="41" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5887,7 +5887,7 @@
         <v>Moreira</v>
       </c>
       <c r="F176" s="45" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -5965,7 +5965,7 @@
         <v>Muller</v>
       </c>
       <c r="F180" s="45" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6064,7 +6064,7 @@
         <v>Nguyen</v>
       </c>
       <c r="F185" s="41" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="186" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6104,7 +6104,7 @@
         <v>Norris</v>
       </c>
       <c r="F187" s="41" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="188" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6144,7 +6144,7 @@
         <v>Ortins</v>
       </c>
       <c r="F189" s="41" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="190" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6205,7 +6205,7 @@
         <v>Patel</v>
       </c>
       <c r="F192" s="46" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6245,7 +6245,7 @@
         <v>Petrin</v>
       </c>
       <c r="F194" s="45" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="195" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6269,7 +6269,7 @@
     </row>
     <row r="196" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A196" s="48" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B196" s="41"/>
       <c r="C196" s="40" t="str">
@@ -6304,7 +6304,7 @@
         <v>Pomerantz</v>
       </c>
       <c r="F197" s="46" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="198" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6325,12 +6325,12 @@
         <v>Poudyal</v>
       </c>
       <c r="F198" s="45" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="199" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A199" s="46" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B199" s="41"/>
       <c r="C199" s="40" t="str">
@@ -6367,7 +6367,7 @@
         <v>Rai</v>
       </c>
       <c r="F200" s="46" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="201" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6445,7 +6445,7 @@
         <v>Richter</v>
       </c>
       <c r="F204" s="46" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="205" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6466,7 +6466,7 @@
         <v>Robichaud</v>
       </c>
       <c r="F205" s="46" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="206" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6582,7 +6582,7 @@
         <v>Rojas</v>
       </c>
       <c r="F211" s="41" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="212" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6606,7 +6606,7 @@
     </row>
     <row r="213" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A213" s="41" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B213" s="41"/>
       <c r="C213" s="40" t="str">
@@ -6643,7 +6643,7 @@
         <v>Sardinha</v>
       </c>
       <c r="F214" s="45" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="215" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6664,7 +6664,7 @@
         <v>Sarre</v>
       </c>
       <c r="F215" s="41" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="216" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6723,7 +6723,7 @@
         <v>Schrager</v>
       </c>
       <c r="F218" s="45" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="219" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6782,12 +6782,12 @@
         <v>Selvakumar</v>
       </c>
       <c r="F221" s="46" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="222" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A222" s="45" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B222" s="41"/>
       <c r="C222" s="40" t="str">
@@ -6841,7 +6841,7 @@
         <v>Shediac</v>
       </c>
       <c r="F224" s="45" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="225" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6881,7 +6881,7 @@
         <v>Siciliano</v>
       </c>
       <c r="F226" s="45" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="227" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -6921,7 +6921,7 @@
         <v>Skenderian</v>
       </c>
       <c r="F228" s="46" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="229" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7001,7 +7001,7 @@
         <v>Soto</v>
       </c>
       <c r="F232" s="45" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="233" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7079,7 +7079,7 @@
         <v>Staffier</v>
       </c>
       <c r="F236" s="46" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="237" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7100,7 +7100,7 @@
         <v>Stathoulopoulos</v>
       </c>
       <c r="F237" s="46" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="238" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7199,7 +7199,7 @@
         <v>Taubman</v>
       </c>
       <c r="F242" s="45" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="243" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7220,7 +7220,7 @@
         <v>Tawadros</v>
       </c>
       <c r="F243" s="41" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="244" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7281,7 +7281,7 @@
         <v>Travassos</v>
       </c>
       <c r="F246" s="45" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="247" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7302,7 +7302,7 @@
         <v>Upton</v>
       </c>
       <c r="F247" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="248" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="D249" s="40"/>
       <c r="E249" s="49" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F249" s="41"/>
     </row>
@@ -7349,10 +7349,10 @@
         <v>Katherine</v>
       </c>
       <c r="D250" s="49" t="s">
+        <v>465</v>
+      </c>
+      <c r="E250" s="49" t="s">
         <v>466</v>
-      </c>
-      <c r="E250" s="49" t="s">
-        <v>467</v>
       </c>
       <c r="F250" s="45"/>
     </row>
@@ -7393,7 +7393,7 @@
         <v>Viliott</v>
       </c>
       <c r="F252" s="45" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="253" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7414,7 +7414,7 @@
         <v>Vitarisi</v>
       </c>
       <c r="F253" s="46" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="254" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -7475,13 +7475,13 @@
       <c r="F256" s="45"/>
     </row>
     <row r="257" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A257" s="46" t="s">
+      <c r="A257" s="45" t="s">
         <v>337</v>
       </c>
       <c r="B257" s="41"/>
       <c r="C257" s="40" t="str">
         <f t="shared" si="12"/>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="D257" s="40" t="str">
         <f t="shared" si="13"/>
@@ -7495,12 +7495,12 @@
     </row>
     <row r="258" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A258" s="45" t="s">
-        <v>338</v>
+        <v>481</v>
       </c>
       <c r="B258" s="41"/>
       <c r="C258" s="40" t="str">
         <f t="shared" si="12"/>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="D258" s="40" t="str">
         <f t="shared" si="13"/>
@@ -7514,7 +7514,7 @@
     </row>
     <row r="259" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A259" s="46" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B259" s="41"/>
       <c r="C259" s="40" t="str">
@@ -7533,7 +7533,7 @@
     </row>
     <row r="260" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A260" s="45" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B260" s="41"/>
       <c r="C260" s="40" t="str">
@@ -7552,7 +7552,7 @@
     </row>
     <row r="261" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A261" s="41" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B261" s="41"/>
       <c r="C261" s="40" t="str">
@@ -7571,7 +7571,7 @@
     </row>
     <row r="262" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A262" s="45" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B262" s="41"/>
       <c r="C262" s="40" t="str">
@@ -7590,7 +7590,7 @@
     </row>
     <row r="263" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A263" s="41" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B263" s="41"/>
       <c r="C263" s="40" t="str">
@@ -7606,12 +7606,12 @@
         <v>Williams</v>
       </c>
       <c r="F263" s="41" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="264" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A264" s="45" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B264" s="41"/>
       <c r="C264" s="40" t="str">
@@ -7630,7 +7630,7 @@
     </row>
     <row r="265" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A265" s="45" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C265" s="40" t="str">
         <f>IF(ISERROR( FIND(",",TRIM(A265))),LEFT(TRIM(A265), FIND(" ",TRIM(A265))-1),MID(TRIM(A265),LEN(C265)+3,FIND(" ",TRIM(A265)&amp;" ",LEN(C265)+3)-LEN(C265)-2))</f>
@@ -7648,7 +7648,7 @@
     </row>
     <row r="266" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A266" s="45" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C266" s="40" t="str">
         <f>IF(ISERROR( FIND(",",TRIM(A266))),LEFT(TRIM(A266), FIND(" ",TRIM(A266))-1),MID(TRIM(A266),LEN(C266)+3,FIND(" ",TRIM(A266)&amp;" ",LEN(C266)+3)-LEN(C266)-2))</f>
@@ -7666,7 +7666,7 @@
     </row>
     <row r="267" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A267" s="41" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C267" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7684,7 +7684,7 @@
     </row>
     <row r="268" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A268" s="45" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C268" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7699,12 +7699,12 @@
         <v>Zani</v>
       </c>
       <c r="F268" s="45" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="269" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A269" s="41" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C269" s="40" t="str">
         <f t="shared" si="15"/>
@@ -7719,7 +7719,7 @@
         <v>Zheng</v>
       </c>
       <c r="F269" s="41" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.2">
@@ -7796,7 +7796,7 @@
       <c r="H2" s="42"/>
       <c r="I2" s="42"/>
       <c r="L2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -7827,7 +7827,7 @@
       <c r="H3" s="42"/>
       <c r="I3" s="42"/>
       <c r="L3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -7858,7 +7858,7 @@
       <c r="H4" s="42"/>
       <c r="I4" s="42"/>
       <c r="L4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -7889,7 +7889,7 @@
       <c r="H5" s="42"/>
       <c r="I5" s="42"/>
       <c r="L5" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -7948,7 +7948,7 @@
       <c r="H7" s="42"/>
       <c r="I7" s="42"/>
       <c r="L7" s="22" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -7982,7 +7982,7 @@
         <v>30</v>
       </c>
       <c r="M8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -8016,7 +8016,7 @@
         <v>87</v>
       </c>
       <c r="M9" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -8050,7 +8050,7 @@
         <v>31</v>
       </c>
       <c r="M10" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -8084,7 +8084,7 @@
         <v>32</v>
       </c>
       <c r="M11" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -8118,7 +8118,7 @@
         <v>33</v>
       </c>
       <c r="M12" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -8152,7 +8152,7 @@
         <v>34</v>
       </c>
       <c r="M13" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -8186,7 +8186,7 @@
         <v>35</v>
       </c>
       <c r="M14" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -8220,7 +8220,7 @@
         <v>36</v>
       </c>
       <c r="M15" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -8254,7 +8254,7 @@
         <v>37</v>
       </c>
       <c r="M16" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -8288,7 +8288,7 @@
         <v>38</v>
       </c>
       <c r="M17" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -8322,7 +8322,7 @@
         <v>39</v>
       </c>
       <c r="M18" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -8356,7 +8356,7 @@
         <v>40</v>
       </c>
       <c r="M19" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -8390,7 +8390,7 @@
         <v>41</v>
       </c>
       <c r="M20" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -8421,10 +8421,10 @@
       <c r="H21" s="42"/>
       <c r="I21" s="42"/>
       <c r="L21" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="M21" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -8455,10 +8455,10 @@
       <c r="H22" s="42"/>
       <c r="I22" s="42"/>
       <c r="L22" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="M22" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -8489,10 +8489,10 @@
       <c r="H23" s="42"/>
       <c r="I23" s="42"/>
       <c r="L23" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M23" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -8526,7 +8526,7 @@
         <v>42</v>
       </c>
       <c r="M24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -10097,7 +10097,7 @@
         <v/>
       </c>
       <c r="E81" s="39" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F81" s="39" t="str">
         <f>'Raw Name Splitter'!F81</f>
@@ -14770,7 +14770,7 @@
         <v>Colby</v>
       </c>
       <c r="E249" s="39" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F249" s="39">
         <f>'Raw Name Splitter'!F249</f>
@@ -14982,7 +14982,7 @@
       </c>
       <c r="C257" s="39" t="str">
         <f>'Raw Name Splitter'!C257</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="D257" s="39" t="str">
         <f>'Raw Name Splitter'!D257</f>
@@ -15010,7 +15010,7 @@
       </c>
       <c r="C258" s="39" t="str">
         <f>'Raw Name Splitter'!C258</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="D258" s="39" t="str">
         <f>'Raw Name Splitter'!D258</f>
@@ -15333,13 +15333,13 @@
         <v>87</v>
       </c>
       <c r="C270" s="39" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E270" s="39" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F270" s="39" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -26133,7 +26133,7 @@
       </c>
       <c r="I248" s="1" t="str">
         <f>VLOOKUP(J248,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="J248">
         <v>235</v>
@@ -26177,7 +26177,7 @@
       </c>
       <c r="I249" s="1" t="str">
         <f>VLOOKUP(J249,'Names with Seat Code'!A:E,3,FALSE)</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="J249">
         <v>236</v>
@@ -36834,7 +36834,7 @@
       </c>
       <c r="H248" s="6" t="str">
         <f>'Grad Raw Data'!I248</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="I248" s="6" t="str">
         <f>'Grad Raw Data'!H248</f>
@@ -36871,7 +36871,7 @@
       </c>
       <c r="H249" s="6" t="str">
         <f>'Grad Raw Data'!I249</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="I249" s="6" t="str">
         <f>'Grad Raw Data'!H249</f>
@@ -48489,7 +48489,7 @@
     <row r="494" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A494" s="20" t="str">
         <f>'Grad Raw Data'!I248</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="B494" s="20" t="str">
         <f>'Grad Raw Data'!K248</f>
@@ -48533,7 +48533,7 @@
     <row r="496" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A496" s="20" t="str">
         <f>'Grad Raw Data'!I249</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="B496" s="20" t="str">
         <f>'Grad Raw Data'!K249</f>
@@ -49123,7 +49123,7 @@
     </row>
     <row r="528" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A528" s="51" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B528" s="50"/>
       <c r="C528" s="20"/>
@@ -56820,7 +56820,7 @@
     <row r="494" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A494" s="20" t="str">
         <f>'Grad Raw Data'!I248</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="B494" s="20" t="str">
         <f>'Grad Raw Data'!K248</f>
@@ -56851,7 +56851,7 @@
     <row r="496" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A496" s="20" t="str">
         <f>'Grad Raw Data'!I249</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="B496" s="20" t="str">
         <f>'Grad Raw Data'!K249</f>
@@ -57249,12 +57249,24 @@
       <c r="F521" s="20"/>
     </row>
     <row r="522" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A522" s="20"/>
+      <c r="A522" s="20" t="str">
+        <f>'Grad Raw Data'!I262</f>
+        <v>Quinn</v>
+      </c>
       <c r="B522" s="20"/>
-      <c r="C522" s="20"/>
+      <c r="C522" s="20" t="str">
+        <f>'Grad Raw Data'!H262</f>
+        <v>Yandle</v>
+      </c>
       <c r="D522" s="20"/>
-      <c r="E522" s="20"/>
-      <c r="F522" s="20"/>
+      <c r="E522" s="20" t="str">
+        <f>'Grad Raw Data'!D264</f>
+        <v>LEFT</v>
+      </c>
+      <c r="F522" s="20">
+        <f>'Grad Raw Data'!E264</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="523" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A523" s="20"/>
@@ -57265,12 +57277,24 @@
       <c r="F523" s="20"/>
     </row>
     <row r="524" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A524" s="20"/>
+      <c r="A524" s="20" t="str">
+        <f>'Grad Raw Data'!I263</f>
+        <v>John</v>
+      </c>
       <c r="B524" s="20"/>
-      <c r="C524" s="20"/>
+      <c r="C524" s="20" t="str">
+        <f>'Grad Raw Data'!H263</f>
+        <v>Zani</v>
+      </c>
       <c r="D524" s="20"/>
-      <c r="E524" s="20"/>
-      <c r="F524" s="20"/>
+      <c r="E524" s="20" t="str">
+        <f>'Grad Raw Data'!D266</f>
+        <v>LEFT</v>
+      </c>
+      <c r="F524" s="20">
+        <f>'Grad Raw Data'!E266</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="525" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A525" s="20"/>
@@ -57281,12 +57305,24 @@
       <c r="F525" s="20"/>
     </row>
     <row r="526" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A526" s="20"/>
+      <c r="A526" s="20" t="str">
+        <f>'Grad Raw Data'!I264</f>
+        <v>Jiayu</v>
+      </c>
       <c r="B526" s="20"/>
-      <c r="C526" s="20"/>
+      <c r="C526" s="20" t="str">
+        <f>'Grad Raw Data'!H264</f>
+        <v>Zheng</v>
+      </c>
       <c r="D526" s="20"/>
-      <c r="E526" s="20"/>
-      <c r="F526" s="20"/>
+      <c r="E526" s="20" t="str">
+        <f>'Grad Raw Data'!D268</f>
+        <v>LEFT</v>
+      </c>
+      <c r="F526" s="20">
+        <f>'Grad Raw Data'!E268</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="527" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A527" s="20"/>
@@ -68060,7 +68096,7 @@
       </c>
       <c r="G321" s="31" t="str">
         <f>VLOOKUP(I321,'Names with Seat Code'!B:E,2)</f>
-        <v>Tess</v>
+        <v>Kyle</v>
       </c>
       <c r="H321" s="31" t="str">
         <f>VLOOKUP(I321,'Names with Seat Code'!B:E,4)</f>
@@ -68092,7 +68128,7 @@
       </c>
       <c r="G322" s="31" t="str">
         <f>VLOOKUP(I322,'Names with Seat Code'!B:E,2)</f>
-        <v>Kyle</v>
+        <v>Tess</v>
       </c>
       <c r="H322" s="31" t="str">
         <f>VLOOKUP(I322,'Names with Seat Code'!B:E,4)</f>

</xml_diff>